<commit_message>
Fix scanner gaps found in review: key files, in-repo --out exclusion, same-line matches
- Route text PEM certificate/key files through the pattern rules after
  metadata parsing so committed private keys produce a redacted Secret row.
- Exclude any --out directory that sits inside the repository, so a second
  scan does not inventory its own JSON/Markdown output.
- Use finditer() per line so minified JSON (root.json) yields one row per
  asset; the TUF key refiner now reads the public value following its own
  match. Inventory grows from 141 to 144 rows (3 additional ECDSA trust keys).
- Regenerate JSON, XLSX, Markdown and PDF.

Co-Authored-By: Erik Rozi <erik.rozi@cognition.ai>
</commit_message>
<xml_diff>
--- a/docs/security/crypto-inventory/Cryptographic-Inventory.xlsx
+++ b/docs/security/crypto-inventory/Cryptographic-Inventory.xlsx
@@ -179,8 +179,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Inventory" displayName="Inventory" ref="A1:V142" headerRowCount="1">
-  <autoFilter ref="A1:V142"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Inventory" displayName="Inventory" ref="A1:V145" headerRowCount="1">
+  <autoFilter ref="A1:V145"/>
   <tableColumns count="22">
     <tableColumn id="1" name="Asset ID"/>
     <tableColumn id="2" name="File"/>
@@ -260,8 +260,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="AgilityGaps" displayName="AgilityGaps" ref="A1:H8" headerRowCount="1">
-  <autoFilter ref="A1:H8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="AgilityGaps" displayName="AgilityGaps" ref="A1:H11" headerRowCount="1">
+  <autoFilter ref="A1:H11"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Asset ID"/>
     <tableColumn id="2" name="File"/>
@@ -277,8 +277,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="MigrationCandidates" displayName="MigrationCandidates" ref="A1:L19" headerRowCount="1">
-  <autoFilter ref="A1:L19"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="MigrationCandidates" displayName="MigrationCandidates" ref="A1:L22" headerRowCount="1">
+  <autoFilter ref="A1:L22"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Asset ID"/>
     <tableColumn id="2" name="Priority"/>
@@ -586,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V142"/>
+  <dimension ref="A1:V145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5949,53 +5949,65 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>api/source/service/STIGService.js</t>
+          <t>root.json</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
-        <v>799</v>
+        <v>1</v>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>API (server)</t>
+          <t>Repository</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Hash</t>
+          <t>Signing</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>SHA-256</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="inlineStr"/>
-      <c r="H58" s="2" t="inlineStr"/>
+          <t>ECDSA (X.509 certificate)</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>secp256r1</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>Certificate subject: [values withheld] attributes: commonName; self-signed (subject = issuer); valid 2021-04-06 to 2031-04-04</t>
+        </is>
+      </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>Content digest used to detect duplicate STIG check/fix text</t>
+          <t>Container image trust metadata (Docker Content Trust / Notary root)</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>node:crypto</t>
-        </is>
-      </c>
-      <c r="K58" s="2" t="inlineStr"/>
+          <t>Notary/TUF (registry)</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>TUF root.json</t>
+        </is>
+      </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>No (deduplication)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>Symmetric — Grover-affected, adequate at ≥256-bit</t>
+          <t>Quantum-vulnerable (Shor)</t>
         </is>
       </c>
       <c r="N58" s="2" t="inlineStr">
         <is>
-          <t>SHA-384 or SHA-512 (already SHA-2; SHA-256 acceptable per CNSA 2.0 where interoperability requires)</t>
+          <t>ML-DSA (FIPS 204) or LMS/XMSS (SP 800-208) for software signing</t>
         </is>
       </c>
       <c r="O58" s="2" t="inlineStr">
@@ -6003,25 +6015,37 @@
           <t>Hardcoded</t>
         </is>
       </c>
-      <c r="P58" s="2" t="inlineStr"/>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>Container registry Notary service and consumer docker clients</t>
+        </is>
+      </c>
       <c r="Q58" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R58" s="2" t="inlineStr">
         <is>
-          <t>Hash function literal in code.</t>
-        </is>
-      </c>
-      <c r="S58" s="2" t="inlineStr"/>
-      <c r="T58" s="2" t="inlineStr"/>
+          <t>Image signature trust roots are ECDSA; verification keys are pinned in this file.</t>
+        </is>
+      </c>
+      <c r="S58" s="2" t="inlineStr">
+        <is>
+          <t>Track registry/Notary support for PQC signatures; re-issue trust roots when available.</t>
+        </is>
+      </c>
+      <c r="T58" s="2" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
       <c r="U58" s="2" t="inlineStr">
         <is>
-          <t>createHash('sha256'</t>
+          <t>"keytype":"ecdsa-x509"</t>
         </is>
       </c>
       <c r="V58" s="2" t="inlineStr">
         <is>
-          <t>HASH-NODE</t>
+          <t>TRUST-TUF-KEY</t>
         </is>
       </c>
     </row>
@@ -6033,53 +6057,61 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>api/source/service/STIGService.js</t>
+          <t>root.json</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
-        <v>802</v>
+        <v>1</v>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>API (server)</t>
+          <t>Repository</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Hash</t>
+          <t>Signing</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>SHA-256</t>
-        </is>
-      </c>
-      <c r="G59" s="2" t="inlineStr"/>
+          <t>ECDSA</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>secp256r1</t>
+        </is>
+      </c>
       <c r="H59" s="2" t="inlineStr"/>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>Content digest used to detect duplicate STIG check/fix text</t>
+          <t>Container image trust metadata (Docker Content Trust / Notary root)</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>node:crypto</t>
-        </is>
-      </c>
-      <c r="K59" s="2" t="inlineStr"/>
+          <t>Notary/TUF (registry)</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>TUF root.json</t>
+        </is>
+      </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>No (deduplication)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="M59" s="2" t="inlineStr">
         <is>
-          <t>Symmetric — Grover-affected, adequate at ≥256-bit</t>
+          <t>Quantum-vulnerable (Shor)</t>
         </is>
       </c>
       <c r="N59" s="2" t="inlineStr">
         <is>
-          <t>SHA-384 or SHA-512 (already SHA-2; SHA-256 acceptable per CNSA 2.0 where interoperability requires)</t>
+          <t>ML-DSA (FIPS 204) or LMS/XMSS (SP 800-208) for software signing</t>
         </is>
       </c>
       <c r="O59" s="2" t="inlineStr">
@@ -6087,25 +6119,37 @@
           <t>Hardcoded</t>
         </is>
       </c>
-      <c r="P59" s="2" t="inlineStr"/>
+      <c r="P59" s="2" t="inlineStr">
+        <is>
+          <t>Container registry Notary service and consumer docker clients</t>
+        </is>
+      </c>
       <c r="Q59" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R59" s="2" t="inlineStr">
         <is>
-          <t>Hash function literal in code.</t>
-        </is>
-      </c>
-      <c r="S59" s="2" t="inlineStr"/>
-      <c r="T59" s="2" t="inlineStr"/>
+          <t>Image signature trust roots are ECDSA; verification keys are pinned in this file.</t>
+        </is>
+      </c>
+      <c r="S59" s="2" t="inlineStr">
+        <is>
+          <t>Track registry/Notary support for PQC signatures; re-issue trust roots when available.</t>
+        </is>
+      </c>
+      <c r="T59" s="2" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
       <c r="U59" s="2" t="inlineStr">
         <is>
-          <t>createHash('sha256'</t>
+          <t>"keytype":"ecdsa"</t>
         </is>
       </c>
       <c r="V59" s="2" t="inlineStr">
         <is>
-          <t>HASH-NODE</t>
+          <t>TRUST-TUF-KEY</t>
         </is>
       </c>
     </row>
@@ -6117,53 +6161,61 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>client/src/js/SM/Attachments.js</t>
+          <t>root.json</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
-        <v>141</v>
+        <v>1</v>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Client (browser)</t>
+          <t>Repository</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Hash</t>
+          <t>Signing</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>SHA-256</t>
-        </is>
-      </c>
-      <c r="G60" s="2" t="inlineStr"/>
+          <t>ECDSA</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>secp256r1</t>
+        </is>
+      </c>
       <c r="H60" s="2" t="inlineStr"/>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>Digest of uploaded attachment stored as metadata (client-computed, not verified server-side)</t>
+          <t>Container image trust metadata (Docker Content Trust / Notary root)</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>Web Crypto (crypto.subtle)</t>
-        </is>
-      </c>
-      <c r="K60" s="2" t="inlineStr"/>
+          <t>Notary/TUF (registry)</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>TUF root.json</t>
+        </is>
+      </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>No (metadata / identification)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>Symmetric — Grover-affected, adequate at ≥256-bit</t>
+          <t>Quantum-vulnerable (Shor)</t>
         </is>
       </c>
       <c r="N60" s="2" t="inlineStr">
         <is>
-          <t>SHA-384 or SHA-512 (already SHA-2; SHA-256 acceptable per CNSA 2.0 where interoperability requires)</t>
+          <t>ML-DSA (FIPS 204) or LMS/XMSS (SP 800-208) for software signing</t>
         </is>
       </c>
       <c r="O60" s="2" t="inlineStr">
@@ -6171,25 +6223,37 @@
           <t>Hardcoded</t>
         </is>
       </c>
-      <c r="P60" s="2" t="inlineStr"/>
+      <c r="P60" s="2" t="inlineStr">
+        <is>
+          <t>Container registry Notary service and consumer docker clients</t>
+        </is>
+      </c>
       <c r="Q60" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R60" s="2" t="inlineStr">
         <is>
-          <t>Hash function literal in browser code.</t>
-        </is>
-      </c>
-      <c r="S60" s="2" t="inlineStr"/>
-      <c r="T60" s="2" t="inlineStr"/>
+          <t>Image signature trust roots are ECDSA; verification keys are pinned in this file.</t>
+        </is>
+      </c>
+      <c r="S60" s="2" t="inlineStr">
+        <is>
+          <t>Track registry/Notary support for PQC signatures; re-issue trust roots when available.</t>
+        </is>
+      </c>
+      <c r="T60" s="2" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
       <c r="U60" s="2" t="inlineStr">
         <is>
-          <t>subtle.digest("SHA-256"</t>
+          <t>"keytype":"ecdsa"</t>
         </is>
       </c>
       <c r="V60" s="2" t="inlineStr">
         <is>
-          <t>HASH-WEBCRYPTO</t>
+          <t>TRUST-TUF-KEY</t>
         </is>
       </c>
     </row>
@@ -6201,15 +6265,15 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>client/src/js/workers/oidc-worker.js</t>
+          <t>api/source/service/STIGService.js</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
-        <v>157</v>
+        <v>799</v>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Client (browser)</t>
+          <t>API (server)</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -6226,22 +6290,18 @@
       <c r="H61" s="2" t="inlineStr"/>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>PKCE code challenge (S256) for the OIDC authorization code flow</t>
+          <t>Content digest used to detect duplicate STIG check/fix text</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>Web Crypto (crypto.subtle)</t>
-        </is>
-      </c>
-      <c r="K61" s="2" t="inlineStr">
-        <is>
-          <t>OAuth 2.0 / PKCE</t>
-        </is>
-      </c>
+          <t>node:crypto</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr"/>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No (deduplication)</t>
         </is>
       </c>
       <c r="M61" s="2" t="inlineStr">
@@ -6265,19 +6325,19 @@
       </c>
       <c r="R61" s="2" t="inlineStr">
         <is>
-          <t>Hash function literal in browser code.</t>
+          <t>Hash function literal in code.</t>
         </is>
       </c>
       <c r="S61" s="2" t="inlineStr"/>
       <c r="T61" s="2" t="inlineStr"/>
       <c r="U61" s="2" t="inlineStr">
         <is>
-          <t>subtle.digest('SHA-256'</t>
+          <t>createHash('sha256'</t>
         </is>
       </c>
       <c r="V61" s="2" t="inlineStr">
         <is>
-          <t>HASH-WEBCRYPTO</t>
+          <t>HASH-NODE</t>
         </is>
       </c>
     </row>
@@ -6289,15 +6349,15 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>client/src/js/workers/oidc-worker.js</t>
+          <t>api/source/service/STIGService.js</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
-        <v>267</v>
+        <v>802</v>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Client (browser)</t>
+          <t>API (server)</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -6307,29 +6367,25 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>SHA-256 (PKCE S256)</t>
+          <t>SHA-256</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr"/>
       <c r="H62" s="2" t="inlineStr"/>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>Bind the OAuth authorization code to the browser client</t>
+          <t>Content digest used to detect duplicate STIG check/fix text</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>Web Crypto (crypto.subtle)</t>
-        </is>
-      </c>
-      <c r="K62" s="2" t="inlineStr">
-        <is>
-          <t>OAuth 2.0 authorization code + PKCE</t>
-        </is>
-      </c>
+          <t>node:crypto</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr"/>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No (deduplication)</t>
         </is>
       </c>
       <c r="M62" s="2" t="inlineStr">
@@ -6347,29 +6403,25 @@
           <t>Hardcoded</t>
         </is>
       </c>
-      <c r="P62" s="2" t="inlineStr">
-        <is>
-          <t>Identity provider must support PKCE S256</t>
-        </is>
-      </c>
+      <c r="P62" s="2" t="inlineStr"/>
       <c r="Q62" s="2" t="n">
         <v>4</v>
       </c>
       <c r="R62" s="2" t="inlineStr">
         <is>
-          <t>SHA-256 commitment; no quantum-vulnerable public-key operation.</t>
+          <t>Hash function literal in code.</t>
         </is>
       </c>
       <c r="S62" s="2" t="inlineStr"/>
       <c r="T62" s="2" t="inlineStr"/>
       <c r="U62" s="2" t="inlineStr">
         <is>
-          <t>code_challenge_method', 'S256'</t>
+          <t>createHash('sha256'</t>
         </is>
       </c>
       <c r="V62" s="2" t="inlineStr">
         <is>
-          <t>OIDC-PKCE-S256</t>
+          <t>HASH-NODE</t>
         </is>
       </c>
     </row>
@@ -6381,15 +6433,15 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>test/utils/mockOidc.js</t>
+          <t>client/src/js/SM/Attachments.js</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
-        <v>37</v>
+        <v>141</v>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Client (browser)</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -6406,18 +6458,18 @@
       <c r="H63" s="2" t="inlineStr"/>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>Derive a JWK key identifier (kid) from the DER public key</t>
+          <t>Digest of uploaded attachment stored as metadata (client-computed, not verified server-side)</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>node:crypto</t>
+          <t>Web Crypto (crypto.subtle)</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>No (identifier)</t>
+          <t>No (metadata / identification)</t>
         </is>
       </c>
       <c r="M63" s="2" t="inlineStr">
@@ -6441,19 +6493,19 @@
       </c>
       <c r="R63" s="2" t="inlineStr">
         <is>
-          <t>Hash function literal in code. Test scope: not deployed.</t>
+          <t>Hash function literal in browser code.</t>
         </is>
       </c>
       <c r="S63" s="2" t="inlineStr"/>
       <c r="T63" s="2" t="inlineStr"/>
       <c r="U63" s="2" t="inlineStr">
         <is>
-          <t>createHash('sha256'</t>
+          <t>subtle.digest("SHA-256"</t>
         </is>
       </c>
       <c r="V63" s="2" t="inlineStr">
         <is>
-          <t>HASH-NODE</t>
+          <t>HASH-WEBCRYPTO</t>
         </is>
       </c>
     </row>
@@ -6465,40 +6517,44 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>.gitignore</t>
+          <t>client/src/js/workers/oidc-worker.js</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
-        <v>26</v>
+        <v>157</v>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Repository</t>
+          <t>Client (browser)</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Certificate/Key material</t>
+          <t>Hash</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Ignored key-material paths</t>
+          <t>SHA-256</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr"/>
       <c r="H64" s="2" t="inlineStr"/>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>Keep PEM files and generated MySQL TLS config out of version control</t>
+          <t>PKCE code challenge (S256) for the OIDC authorization code flow</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>git</t>
-        </is>
-      </c>
-      <c r="K64" s="2" t="inlineStr"/>
+          <t>Web Crypto (crypto.subtle)</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>OAuth 2.0 / PKCE</t>
+        </is>
+      </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -6506,17 +6562,17 @@
       </c>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>Not applicable (no quantum-relevant primitive)</t>
+          <t>Symmetric — Grover-affected, adequate at ≥256-bit</t>
         </is>
       </c>
       <c r="N64" s="2" t="inlineStr">
         <is>
-          <t>None required</t>
+          <t>SHA-384 or SHA-512 (already SHA-2; SHA-256 acceptable per CNSA 2.0 where interoperability requires)</t>
         </is>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Hardcoded</t>
         </is>
       </c>
       <c r="P64" s="2" t="inlineStr"/>
@@ -6525,19 +6581,19 @@
       </c>
       <c r="R64" s="2" t="inlineStr">
         <is>
-          <t>Explains why no certificate or key files are tracked in the repository. 5 occurrences in this file; first occurrence listed.</t>
+          <t>Hash function literal in browser code.</t>
         </is>
       </c>
       <c r="S64" s="2" t="inlineStr"/>
       <c r="T64" s="2" t="inlineStr"/>
       <c r="U64" s="2" t="inlineStr">
         <is>
-          <t>**.pem</t>
+          <t>subtle.digest('SHA-256'</t>
         </is>
       </c>
       <c r="V64" s="2" t="inlineStr">
         <is>
-          <t>KEYMAT-GITIGNORE</t>
+          <t>HASH-WEBCRYPTO</t>
         </is>
       </c>
     </row>
@@ -6549,44 +6605,44 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/api-audit-test-coverage-response.yml</t>
+          <t>client/src/js/workers/oidc-worker.js</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
-        <v>49</v>
+        <v>267</v>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>Client (browser)</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Runtime</t>
+          <t>Hash</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Node.js runtime (CI)</t>
-        </is>
-      </c>
-      <c r="G65" s="2" t="inlineStr">
-        <is>
-          <t>lts/*</t>
-        </is>
-      </c>
+          <t>SHA-256 (PKCE S256)</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr"/>
       <c r="H65" s="2" t="inlineStr"/>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>Node used for CI test runs</t>
+          <t>Bind the OAuth authorization code to the browser client</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>actions/setup-node</t>
-        </is>
-      </c>
-      <c r="K65" s="2" t="inlineStr"/>
+          <t>Web Crypto (crypto.subtle)</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>OAuth 2.0 authorization code + PKCE</t>
+        </is>
+      </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -6594,38 +6650,42 @@
       </c>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>Not applicable (no quantum-relevant primitive)</t>
+          <t>Symmetric — Grover-affected, adequate at ≥256-bit</t>
         </is>
       </c>
       <c r="N65" s="2" t="inlineStr">
         <is>
-          <t>None required</t>
+          <t>SHA-384 or SHA-512 (already SHA-2; SHA-256 acceptable per CNSA 2.0 where interoperability requires)</t>
         </is>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>Configurable</t>
-        </is>
-      </c>
-      <c r="P65" s="2" t="inlineStr"/>
+          <t>Hardcoded</t>
+        </is>
+      </c>
+      <c r="P65" s="2" t="inlineStr">
+        <is>
+          <t>Identity provider must support PKCE S256</t>
+        </is>
+      </c>
       <c r="Q65" s="2" t="n">
         <v>4</v>
       </c>
       <c r="R65" s="2" t="inlineStr">
         <is>
-          <t>CI alias resolves to the current LTS at run time.</t>
+          <t>SHA-256 commitment; no quantum-vulnerable public-key operation.</t>
         </is>
       </c>
       <c r="S65" s="2" t="inlineStr"/>
       <c r="T65" s="2" t="inlineStr"/>
       <c r="U65" s="2" t="inlineStr">
         <is>
-          <t>node-version: lts/*</t>
+          <t>code_challenge_method', 'S256'</t>
         </is>
       </c>
       <c r="V65" s="2" t="inlineStr">
         <is>
-          <t>RUNTIME-CI-NODE</t>
+          <t>OIDC-PKCE-S256</t>
         </is>
       </c>
     </row>
@@ -6637,62 +6697,58 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/api-binary-tests.yml</t>
+          <t>test/utils/mockOidc.js</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Runtime</t>
+          <t>Hash</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Node.js runtime (CI)</t>
-        </is>
-      </c>
-      <c r="G66" s="2" t="inlineStr">
-        <is>
-          <t>lts/*</t>
-        </is>
-      </c>
+          <t>SHA-256</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr"/>
       <c r="H66" s="2" t="inlineStr"/>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>Node used for CI test runs</t>
+          <t>Derive a JWK key identifier (kid) from the DER public key</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>actions/setup-node</t>
+          <t>node:crypto</t>
         </is>
       </c>
       <c r="K66" s="2" t="inlineStr"/>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No (identifier)</t>
         </is>
       </c>
       <c r="M66" s="2" t="inlineStr">
         <is>
-          <t>Not applicable (no quantum-relevant primitive)</t>
+          <t>Symmetric — Grover-affected, adequate at ≥256-bit</t>
         </is>
       </c>
       <c r="N66" s="2" t="inlineStr">
         <is>
-          <t>None required</t>
+          <t>SHA-384 or SHA-512 (already SHA-2; SHA-256 acceptable per CNSA 2.0 where interoperability requires)</t>
         </is>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>Configurable</t>
+          <t>Hardcoded</t>
         </is>
       </c>
       <c r="P66" s="2" t="inlineStr"/>
@@ -6701,19 +6757,19 @@
       </c>
       <c r="R66" s="2" t="inlineStr">
         <is>
-          <t>CI alias resolves to the current LTS at run time.</t>
+          <t>Hash function literal in code. Test scope: not deployed.</t>
         </is>
       </c>
       <c r="S66" s="2" t="inlineStr"/>
       <c r="T66" s="2" t="inlineStr"/>
       <c r="U66" s="2" t="inlineStr">
         <is>
-          <t>node-version: lts/*</t>
+          <t>createHash('sha256'</t>
         </is>
       </c>
       <c r="V66" s="2" t="inlineStr">
         <is>
-          <t>RUNTIME-CI-NODE</t>
+          <t>HASH-NODE</t>
         </is>
       </c>
     </row>
@@ -6725,41 +6781,37 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/api-binary-tests.yml</t>
+          <t>.gitignore</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
-        <v>94</v>
+        <v>26</v>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>Repository</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Runtime</t>
+          <t>Certificate/Key material</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Node.js runtime (CI)</t>
-        </is>
-      </c>
-      <c r="G67" s="2" t="inlineStr">
-        <is>
-          <t>lts/*</t>
-        </is>
-      </c>
+          <t>Ignored key-material paths</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr"/>
       <c r="H67" s="2" t="inlineStr"/>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>Node used for CI test runs</t>
+          <t>Keep PEM files and generated MySQL TLS config out of version control</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>actions/setup-node</t>
+          <t>git</t>
         </is>
       </c>
       <c r="K67" s="2" t="inlineStr"/>
@@ -6780,7 +6832,7 @@
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>Configurable</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="P67" s="2" t="inlineStr"/>
@@ -6789,19 +6841,19 @@
       </c>
       <c r="R67" s="2" t="inlineStr">
         <is>
-          <t>CI alias resolves to the current LTS at run time.</t>
+          <t>Explains why no certificate or key files are tracked in the repository. 5 occurrences in this file; first occurrence listed.</t>
         </is>
       </c>
       <c r="S67" s="2" t="inlineStr"/>
       <c r="T67" s="2" t="inlineStr"/>
       <c r="U67" s="2" t="inlineStr">
         <is>
-          <t>node-version: lts/*</t>
+          <t>**.pem</t>
         </is>
       </c>
       <c r="V67" s="2" t="inlineStr">
         <is>
-          <t>RUNTIME-CI-NODE</t>
+          <t>KEYMAT-GITIGNORE</t>
         </is>
       </c>
     </row>
@@ -6813,11 +6865,11 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/api-container-tests.yml</t>
+          <t>.github/workflows/api-audit-test-coverage-response.yml</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
@@ -6831,23 +6883,23 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Node.js runtime (container test matrix)</t>
+          <t>Node.js runtime (CI)</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>node:lts-alpine</t>
+          <t>lts/*</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>Base image used to build the API container in CI</t>
+          <t>Node used for CI test runs</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>Docker</t>
+          <t>actions/setup-node</t>
         </is>
       </c>
       <c r="K68" s="2" t="inlineStr"/>
@@ -6858,12 +6910,12 @@
       </c>
       <c r="M68" s="2" t="inlineStr">
         <is>
-          <t>Protocol/configuration — inherits class of negotiated algorithms</t>
+          <t>Not applicable (no quantum-relevant primitive)</t>
         </is>
       </c>
       <c r="N68" s="2" t="inlineStr">
         <is>
-          <t>TLS 1.3 with ML-KEM key establishment and ML-DSA certificates when available</t>
+          <t>None required</t>
         </is>
       </c>
       <c r="O68" s="2" t="inlineStr">
@@ -6873,23 +6925,23 @@
       </c>
       <c r="P68" s="2" t="inlineStr"/>
       <c r="Q68" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R68" s="2" t="inlineStr">
         <is>
-          <t>Same mutable tag as the Dockerfile default.</t>
+          <t>CI alias resolves to the current LTS at run time.</t>
         </is>
       </c>
       <c r="S68" s="2" t="inlineStr"/>
       <c r="T68" s="2" t="inlineStr"/>
       <c r="U68" s="2" t="inlineStr">
         <is>
-          <t>build_arg: "node:lts-alpine"</t>
+          <t>node-version: lts/*</t>
         </is>
       </c>
       <c r="V68" s="2" t="inlineStr">
         <is>
-          <t>RUNTIME-CI-CONTAINER-ARG</t>
+          <t>RUNTIME-CI-NODE</t>
         </is>
       </c>
     </row>
@@ -6901,11 +6953,11 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/api-spec-validation.yml</t>
+          <t>.github/workflows/api-binary-tests.yml</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
@@ -6989,11 +7041,11 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/unit-tests.yml</t>
+          <t>.github/workflows/api-binary-tests.yml</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
-        <v>27</v>
+        <v>94</v>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
@@ -7077,15 +7129,15 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Dockerfile</t>
+          <t>.github/workflows/api-container-tests.yml</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Repository</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -7095,7 +7147,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Node.js/OpenSSL runtime (container base image)</t>
+          <t>Node.js runtime (container test matrix)</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -7106,12 +7158,12 @@
       <c r="H71" s="2" t="inlineStr"/>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>Provides the TLS stack and node:crypto for the API</t>
+          <t>Base image used to build the API container in CI</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>Container base image</t>
+          <t>Docker</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -7135,37 +7187,25 @@
           <t>Configurable</t>
         </is>
       </c>
-      <c r="P71" s="2" t="inlineStr">
-        <is>
-          <t>Upstream Node.js image publisher (mutable tag)</t>
-        </is>
-      </c>
+      <c r="P71" s="2" t="inlineStr"/>
       <c r="Q71" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R71" s="2" t="inlineStr">
         <is>
-          <t>Tag is mutable; the OpenSSL version that decides ML-KEM/ML-DSA availability is not pinned.</t>
-        </is>
-      </c>
-      <c r="S71" s="2" t="inlineStr">
-        <is>
-          <t>Pin a specific Node.js LTS major (24.x) with OpenSSL 3.5+ and record it in the inventory on each release.</t>
-        </is>
-      </c>
-      <c r="T71" s="2" t="inlineStr">
-        <is>
-          <t>Phase 0 / Phase 1</t>
-        </is>
-      </c>
+          <t>Same mutable tag as the Dockerfile default.</t>
+        </is>
+      </c>
+      <c r="S71" s="2" t="inlineStr"/>
+      <c r="T71" s="2" t="inlineStr"/>
       <c r="U71" s="2" t="inlineStr">
         <is>
-          <t>ARG BASE_IMAGE="node:lts-alpine"</t>
+          <t>build_arg: "node:lts-alpine"</t>
         </is>
       </c>
       <c r="V71" s="2" t="inlineStr">
         <is>
-          <t>RUNTIME-DOCKER-BASE</t>
+          <t>RUNTIME-CI-CONTAINER-ARG</t>
         </is>
       </c>
     </row>
@@ -7177,15 +7217,15 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>api/pkg.config.json</t>
+          <t>.github/workflows/api-spec-validation.yml</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>API (server)</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -7195,23 +7235,23 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Node.js runtime (packaged binaries)</t>
+          <t>Node.js runtime (CI)</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>node24-win,node24-linuxstatic</t>
+          <t>lts/*</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>Node major embedded in the standalone API binaries</t>
+          <t>Node used for CI test runs</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>@yao-pkg/pkg</t>
+          <t>actions/setup-node</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr"/>
@@ -7222,12 +7262,12 @@
       </c>
       <c r="M72" s="2" t="inlineStr">
         <is>
-          <t>Protocol/configuration — inherits class of negotiated algorithms</t>
+          <t>Not applicable (no quantum-relevant primitive)</t>
         </is>
       </c>
       <c r="N72" s="2" t="inlineStr">
         <is>
-          <t>TLS 1.3 with ML-KEM key establishment and ML-DSA certificates when available</t>
+          <t>None required</t>
         </is>
       </c>
       <c r="O72" s="2" t="inlineStr">
@@ -7237,23 +7277,23 @@
       </c>
       <c r="P72" s="2" t="inlineStr"/>
       <c r="Q72" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R72" s="2" t="inlineStr">
         <is>
-          <t>Binary releases embed a Node 24 runtime; the exact OpenSSL build is fixed at packaging time.</t>
+          <t>CI alias resolves to the current LTS at run time.</t>
         </is>
       </c>
       <c r="S72" s="2" t="inlineStr"/>
       <c r="T72" s="2" t="inlineStr"/>
       <c r="U72" s="2" t="inlineStr">
         <is>
-          <t>"targets": ["node24-win", "node24-linuxstatic"]</t>
+          <t>node-version: lts/*</t>
         </is>
       </c>
       <c r="V72" s="2" t="inlineStr">
         <is>
-          <t>RUNTIME-PKG-TARGET</t>
+          <t>RUNTIME-CI-NODE</t>
         </is>
       </c>
     </row>
@@ -7265,15 +7305,15 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>docs/Dockerfile</t>
+          <t>.github/workflows/unit-tests.yml</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
@@ -7283,23 +7323,23 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Container base image (build tooling; no deployed runtime crypto role)</t>
+          <t>Node.js runtime (CI)</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>sphinxdoc/sphinx:7.4.7</t>
+          <t>lts/*</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr"/>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>Provides the TLS stack and node:crypto for the API</t>
+          <t>Node used for CI test runs</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>Container base image</t>
+          <t>actions/setup-node</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr"/>
@@ -7329,19 +7369,19 @@
       </c>
       <c r="R73" s="2" t="inlineStr">
         <is>
-          <t>Documentation build image; not part of the deployed system.</t>
+          <t>CI alias resolves to the current LTS at run time.</t>
         </is>
       </c>
       <c r="S73" s="2" t="inlineStr"/>
       <c r="T73" s="2" t="inlineStr"/>
       <c r="U73" s="2" t="inlineStr">
         <is>
-          <t>FROM sphinxdoc/sphinx:7.4.7</t>
+          <t>node-version: lts/*</t>
         </is>
       </c>
       <c r="V73" s="2" t="inlineStr">
         <is>
-          <t>RUNTIME-DOCKER-BASE</t>
+          <t>RUNTIME-CI-NODE</t>
         </is>
       </c>
     </row>
@@ -7353,79 +7393,95 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>client/src/js/init.js</t>
+          <t>Dockerfile</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
-        <v>226</v>
+        <v>15</v>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Client (browser)</t>
+          <t>Repository</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Randomness</t>
+          <t>Runtime</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>CSPRNG (platform)</t>
-        </is>
-      </c>
-      <c r="G74" s="2" t="inlineStr"/>
+          <t>Node.js/OpenSSL runtime (container base image)</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>node:lts-alpine</t>
+        </is>
+      </c>
       <c r="H74" s="2" t="inlineStr"/>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>Identifier generation (UUID)</t>
+          <t>Provides the TLS stack and node:crypto for the API</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>node:crypto / Web Crypto</t>
+          <t>Container base image</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
       <c r="L74" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="M74" s="2" t="inlineStr">
         <is>
-          <t>Not applicable (no quantum-relevant primitive)</t>
+          <t>Protocol/configuration — inherits class of negotiated algorithms</t>
         </is>
       </c>
       <c r="N74" s="2" t="inlineStr">
         <is>
-          <t>None required</t>
+          <t>TLS 1.3 with ML-KEM key establishment and ML-DSA certificates when available</t>
         </is>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="P74" s="2" t="inlineStr"/>
+          <t>Configurable</t>
+        </is>
+      </c>
+      <c r="P74" s="2" t="inlineStr">
+        <is>
+          <t>Upstream Node.js image publisher (mutable tag)</t>
+        </is>
+      </c>
       <c r="Q74" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R74" s="2" t="inlineStr">
         <is>
-          <t>Randomness source; not affected by Shor or Grover in a way that changes the migration plan.</t>
-        </is>
-      </c>
-      <c r="S74" s="2" t="inlineStr"/>
-      <c r="T74" s="2" t="inlineStr"/>
+          <t>Tag is mutable; the OpenSSL version that decides ML-KEM/ML-DSA availability is not pinned.</t>
+        </is>
+      </c>
+      <c r="S74" s="2" t="inlineStr">
+        <is>
+          <t>Pin a specific Node.js LTS major (24.x) with OpenSSL 3.5+ and record it in the inventory on each release.</t>
+        </is>
+      </c>
+      <c r="T74" s="2" t="inlineStr">
+        <is>
+          <t>Phase 0 / Phase 1</t>
+        </is>
+      </c>
       <c r="U74" s="2" t="inlineStr">
         <is>
-          <t>crypto.randomUUID(</t>
+          <t>ARG BASE_IMAGE="node:lts-alpine"</t>
         </is>
       </c>
       <c r="V74" s="2" t="inlineStr">
         <is>
-          <t>RNG-CSPRNG</t>
+          <t>RUNTIME-DOCKER-BASE</t>
         </is>
       </c>
     </row>
@@ -7437,37 +7493,41 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>client/src/js/init.js</t>
+          <t>api/pkg.config.json</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
-        <v>256</v>
+        <v>14</v>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Client (browser)</t>
+          <t>API (server)</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Randomness</t>
+          <t>Runtime</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>CSPRNG (platform)</t>
-        </is>
-      </c>
-      <c r="G75" s="2" t="inlineStr"/>
+          <t>Node.js runtime (packaged binaries)</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>node24-win,node24-linuxstatic</t>
+        </is>
+      </c>
       <c r="H75" s="2" t="inlineStr"/>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>OAuth state/nonce generation</t>
+          <t>Node major embedded in the standalone API binaries</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr">
         <is>
-          <t>node:crypto / Web Crypto</t>
+          <t>@yao-pkg/pkg</t>
         </is>
       </c>
       <c r="K75" s="2" t="inlineStr"/>
@@ -7478,38 +7538,38 @@
       </c>
       <c r="M75" s="2" t="inlineStr">
         <is>
-          <t>Not applicable (no quantum-relevant primitive)</t>
+          <t>Protocol/configuration — inherits class of negotiated algorithms</t>
         </is>
       </c>
       <c r="N75" s="2" t="inlineStr">
         <is>
-          <t>None required</t>
+          <t>TLS 1.3 with ML-KEM key establishment and ML-DSA certificates when available</t>
         </is>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Configurable</t>
         </is>
       </c>
       <c r="P75" s="2" t="inlineStr"/>
       <c r="Q75" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R75" s="2" t="inlineStr">
         <is>
-          <t>Randomness source; not affected by Shor or Grover in a way that changes the migration plan.</t>
+          <t>Binary releases embed a Node 24 runtime; the exact OpenSSL build is fixed at packaging time.</t>
         </is>
       </c>
       <c r="S75" s="2" t="inlineStr"/>
       <c r="T75" s="2" t="inlineStr"/>
       <c r="U75" s="2" t="inlineStr">
         <is>
-          <t>crypto.randomUUID(</t>
+          <t>"targets": ["node24-win", "node24-linuxstatic"]</t>
         </is>
       </c>
       <c r="V75" s="2" t="inlineStr">
         <is>
-          <t>RNG-CSPRNG</t>
+          <t>RUNTIME-PKG-TARGET</t>
         </is>
       </c>
     </row>
@@ -7521,43 +7581,47 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>client/src/js/workers/oidc-worker.js</t>
+          <t>docs/Dockerfile</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Client (browser)</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Randomness</t>
+          <t>Runtime</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>CSPRNG (platform)</t>
-        </is>
-      </c>
-      <c r="G76" s="2" t="inlineStr"/>
+          <t>Container base image (build tooling; no deployed runtime crypto role)</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>sphinxdoc/sphinx:7.4.7</t>
+        </is>
+      </c>
       <c r="H76" s="2" t="inlineStr"/>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>BroadcastChannel name</t>
+          <t>Provides the TLS stack and node:crypto for the API</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>node:crypto / Web Crypto</t>
+          <t>Container base image</t>
         </is>
       </c>
       <c r="K76" s="2" t="inlineStr"/>
       <c r="L76" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="M76" s="2" t="inlineStr">
@@ -7572,7 +7636,7 @@
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Configurable</t>
         </is>
       </c>
       <c r="P76" s="2" t="inlineStr"/>
@@ -7581,19 +7645,19 @@
       </c>
       <c r="R76" s="2" t="inlineStr">
         <is>
-          <t>Randomness source; not affected by Shor or Grover in a way that changes the migration plan.</t>
+          <t>Documentation build image; not part of the deployed system.</t>
         </is>
       </c>
       <c r="S76" s="2" t="inlineStr"/>
       <c r="T76" s="2" t="inlineStr"/>
       <c r="U76" s="2" t="inlineStr">
         <is>
-          <t>crypto.randomUUID(</t>
+          <t>FROM sphinxdoc/sphinx:7.4.7</t>
         </is>
       </c>
       <c r="V76" s="2" t="inlineStr">
         <is>
-          <t>RNG-CSPRNG</t>
+          <t>RUNTIME-DOCKER-BASE</t>
         </is>
       </c>
     </row>
@@ -7605,11 +7669,11 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>client/src/js/workers/oidc-worker.js</t>
+          <t>client/src/js/init.js</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
-        <v>150</v>
+        <v>226</v>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
@@ -7630,7 +7694,7 @@
       <c r="H77" s="2" t="inlineStr"/>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>PKCE code verifier generation</t>
+          <t>Identifier generation (UUID)</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr">
@@ -7641,7 +7705,7 @@
       <c r="K77" s="2" t="inlineStr"/>
       <c r="L77" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="M77" s="2" t="inlineStr">
@@ -7665,14 +7729,14 @@
       </c>
       <c r="R77" s="2" t="inlineStr">
         <is>
-          <t>Randomness source; not affected by Shor or Grover in a way that changes the migration plan. 3 occurrences in this file; first occurrence listed.</t>
+          <t>Randomness source; not affected by Shor or Grover in a way that changes the migration plan.</t>
         </is>
       </c>
       <c r="S77" s="2" t="inlineStr"/>
       <c r="T77" s="2" t="inlineStr"/>
       <c r="U77" s="2" t="inlineStr">
         <is>
-          <t>crypto.getRandomValues(</t>
+          <t>crypto.randomUUID(</t>
         </is>
       </c>
       <c r="V77" s="2" t="inlineStr">
@@ -7689,11 +7753,11 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>client/src/js/workers/state-worker.js</t>
+          <t>client/src/js/init.js</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
-        <v>13</v>
+        <v>256</v>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
@@ -7773,11 +7837,11 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>client/src/reauth.html</t>
+          <t>client/src/js/workers/oidc-worker.js</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
@@ -7798,7 +7862,7 @@
       <c r="H79" s="2" t="inlineStr"/>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>Identifier generation (UUID)</t>
+          <t>BroadcastChannel name</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr">
@@ -7857,15 +7921,15 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>test/utils/mockOidc.js</t>
+          <t>client/src/js/workers/oidc-worker.js</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Client (browser)</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -7882,7 +7946,7 @@
       <c r="H80" s="2" t="inlineStr"/>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>Identifier generation (UUID)</t>
+          <t>PKCE code verifier generation</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -7893,7 +7957,7 @@
       <c r="K80" s="2" t="inlineStr"/>
       <c r="L80" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="M80" s="2" t="inlineStr">
@@ -7917,14 +7981,14 @@
       </c>
       <c r="R80" s="2" t="inlineStr">
         <is>
-          <t>Randomness source; not affected by Shor or Grover in a way that changes the migration plan. 4 occurrences in this file; first occurrence listed. Test scope: not deployed.</t>
+          <t>Randomness source; not affected by Shor or Grover in a way that changes the migration plan. 3 occurrences in this file; first occurrence listed.</t>
         </is>
       </c>
       <c r="S80" s="2" t="inlineStr"/>
       <c r="T80" s="2" t="inlineStr"/>
       <c r="U80" s="2" t="inlineStr">
         <is>
-          <t>randomBytes(</t>
+          <t>crypto.getRandomValues(</t>
         </is>
       </c>
       <c r="V80" s="2" t="inlineStr">
@@ -7941,35 +8005,39 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/api-audit-test-coverage-response.yml</t>
+          <t>client/src/js/workers/state-worker.js</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>Client (browser)</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Secret</t>
+          <t>Randomness</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Database password literal (STIGMAN_DB_PASSWORD)</t>
+          <t>CSPRNG (platform)</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr"/>
       <c r="H81" s="2" t="inlineStr"/>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>Credential literal (type: database password)</t>
-        </is>
-      </c>
-      <c r="J81" s="2" t="inlineStr"/>
+          <t>OAuth state/nonce generation</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>node:crypto / Web Crypto</t>
+        </is>
+      </c>
       <c r="K81" s="2" t="inlineStr"/>
       <c r="L81" s="2" t="inlineStr">
         <is>
@@ -7988,28 +8056,28 @@
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>Hardcoded</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="P81" s="2" t="inlineStr"/>
       <c r="Q81" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R81" s="2" t="inlineStr">
         <is>
-          <t>Literal credential in test/CI configuration; must not be reused in production.</t>
+          <t>Randomness source; not affected by Shor or Grover in a way that changes the migration plan.</t>
         </is>
       </c>
       <c r="S81" s="2" t="inlineStr"/>
       <c r="T81" s="2" t="inlineStr"/>
       <c r="U81" s="2" t="inlineStr">
         <is>
-          <t>[redacted] database password literal</t>
+          <t>crypto.randomUUID(</t>
         </is>
       </c>
       <c r="V81" s="2" t="inlineStr">
         <is>
-          <t>SECRET-DB-PASSWORD-LITERAL</t>
+          <t>RNG-CSPRNG</t>
         </is>
       </c>
     </row>
@@ -8021,39 +8089,43 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/api-audit-test-coverage-response.yml</t>
+          <t>client/src/reauth.html</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
-        <v>71</v>
+        <v>33</v>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>Client (browser)</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Secret</t>
+          <t>Randomness</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Database password literal (MYSQL_ROOT_PASSWORD)</t>
+          <t>CSPRNG (platform)</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr"/>
       <c r="H82" s="2" t="inlineStr"/>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>Credential literal (type: database password)</t>
-        </is>
-      </c>
-      <c r="J82" s="2" t="inlineStr"/>
+          <t>Identifier generation (UUID)</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>node:crypto / Web Crypto</t>
+        </is>
+      </c>
       <c r="K82" s="2" t="inlineStr"/>
       <c r="L82" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="M82" s="2" t="inlineStr">
@@ -8068,28 +8140,28 @@
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>Hardcoded</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="P82" s="2" t="inlineStr"/>
       <c r="Q82" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R82" s="2" t="inlineStr">
         <is>
-          <t>Literal credential in test/CI configuration; must not be reused in production.</t>
+          <t>Randomness source; not affected by Shor or Grover in a way that changes the migration plan.</t>
         </is>
       </c>
       <c r="S82" s="2" t="inlineStr"/>
       <c r="T82" s="2" t="inlineStr"/>
       <c r="U82" s="2" t="inlineStr">
         <is>
-          <t>[redacted] database password literal</t>
+          <t>crypto.randomUUID(</t>
         </is>
       </c>
       <c r="V82" s="2" t="inlineStr">
         <is>
-          <t>SECRET-DB-PASSWORD-LITERAL</t>
+          <t>RNG-CSPRNG</t>
         </is>
       </c>
     </row>
@@ -8101,39 +8173,43 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/api-audit-test-coverage-response.yml</t>
+          <t>test/utils/mockOidc.js</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
-        <v>74</v>
+        <v>159</v>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Secret</t>
+          <t>Randomness</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Database password literal (MYSQL_PASSWORD)</t>
+          <t>CSPRNG (platform)</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr"/>
       <c r="H83" s="2" t="inlineStr"/>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>Credential literal (type: database password)</t>
-        </is>
-      </c>
-      <c r="J83" s="2" t="inlineStr"/>
+          <t>Identifier generation (UUID)</t>
+        </is>
+      </c>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>node:crypto / Web Crypto</t>
+        </is>
+      </c>
       <c r="K83" s="2" t="inlineStr"/>
       <c r="L83" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="M83" s="2" t="inlineStr">
@@ -8148,28 +8224,28 @@
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>Hardcoded</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="P83" s="2" t="inlineStr"/>
       <c r="Q83" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R83" s="2" t="inlineStr">
         <is>
-          <t>Literal credential in test/CI configuration; must not be reused in production.</t>
+          <t>Randomness source; not affected by Shor or Grover in a way that changes the migration plan. 4 occurrences in this file; first occurrence listed. Test scope: not deployed.</t>
         </is>
       </c>
       <c r="S83" s="2" t="inlineStr"/>
       <c r="T83" s="2" t="inlineStr"/>
       <c r="U83" s="2" t="inlineStr">
         <is>
-          <t>[redacted] database password literal</t>
+          <t>randomBytes(</t>
         </is>
       </c>
       <c r="V83" s="2" t="inlineStr">
         <is>
-          <t>SECRET-DB-PASSWORD-LITERAL</t>
+          <t>RNG-CSPRNG</t>
         </is>
       </c>
     </row>
@@ -8181,11 +8257,11 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/api-binary-tests.yml</t>
+          <t>.github/workflows/api-audit-test-coverage-response.yml</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
@@ -8261,11 +8337,11 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/api-binary-tests.yml</t>
+          <t>.github/workflows/api-audit-test-coverage-response.yml</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
-        <v>107</v>
+        <v>71</v>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
@@ -8341,11 +8417,11 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/api-binary-tests.yml</t>
+          <t>.github/workflows/api-audit-test-coverage-response.yml</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
-        <v>110</v>
+        <v>74</v>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
@@ -8421,11 +8497,11 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/api-container-tests.yml</t>
+          <t>.github/workflows/api-binary-tests.yml</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
@@ -8439,7 +8515,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Database password literal (MYSQL_ROOT_PASSWORD)</t>
+          <t>Database password literal (STIGMAN_DB_PASSWORD)</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr"/>
@@ -8501,11 +8577,11 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/api-container-tests.yml</t>
+          <t>.github/workflows/api-binary-tests.yml</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
-        <v>62</v>
+        <v>107</v>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
@@ -8519,7 +8595,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>Database password literal (MYSQL_PASSWORD)</t>
+          <t>Database password literal (MYSQL_ROOT_PASSWORD)</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr"/>
@@ -8581,11 +8657,11 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/api-container-tests.yml</t>
+          <t>.github/workflows/api-binary-tests.yml</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
-        <v>72</v>
+        <v>110</v>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
@@ -8599,7 +8675,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>Database password literal (STIGMAN_DB_PASSWORD)</t>
+          <t>Database password literal (MYSQL_PASSWORD)</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr"/>
@@ -8661,15 +8737,15 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>docs/the-project/DockerHub_Readme.md</t>
+          <t>.github/workflows/api-container-tests.yml</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -8741,15 +8817,15 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>docs/the-project/DockerHub_Readme.md</t>
+          <t>.github/workflows/api-container-tests.yml</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -8821,15 +8897,15 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>docs/the-project/DockerHub_Readme.md</t>
+          <t>.github/workflows/api-container-tests.yml</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -8905,7 +8981,7 @@
         </is>
       </c>
       <c r="C93" s="2" t="n">
-        <v>109</v>
+        <v>45</v>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
@@ -8985,7 +9061,7 @@
         </is>
       </c>
       <c r="C94" s="2" t="n">
-        <v>112</v>
+        <v>47</v>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
@@ -9061,15 +9137,15 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>test/api/README.md</t>
+          <t>docs/the-project/DockerHub_Readme.md</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -9079,7 +9155,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>Database password literal (MYSQL_ROOT_PASSWORD)</t>
+          <t>Database password literal (STIGMAN_DB_PASSWORD)</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr"/>
@@ -9141,15 +9217,15 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>test/api/README.md</t>
+          <t>docs/the-project/DockerHub_Readme.md</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
-        <v>32</v>
+        <v>109</v>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -9159,7 +9235,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>Database password literal (MYSQL_PASSWORD)</t>
+          <t>Database password literal (MYSQL_ROOT_PASSWORD)</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
@@ -9221,15 +9297,15 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>test/api/mocha/cross-boundary/lvl1.test.js</t>
+          <t>docs/the-project/DockerHub_Readme.md</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
-        <v>14</v>
+        <v>112</v>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
@@ -9239,14 +9315,14 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>JWT literal</t>
+          <t>Database password literal (MYSQL_PASSWORD)</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr"/>
       <c r="H97" s="2" t="inlineStr"/>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>Embedded signed token (type: bearer token fixture)</t>
+          <t>Credential literal (type: database password)</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr"/>
@@ -9273,23 +9349,23 @@
       </c>
       <c r="P97" s="2" t="inlineStr"/>
       <c r="Q97" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R97" s="2" t="inlineStr">
         <is>
-          <t>Test fixture tokens; they are signed with test keys and expire. 2 occurrences in this file; first occurrence listed.</t>
+          <t>Literal credential in test/CI configuration; must not be reused in production.</t>
         </is>
       </c>
       <c r="S97" s="2" t="inlineStr"/>
       <c r="T97" s="2" t="inlineStr"/>
       <c r="U97" s="2" t="inlineStr">
         <is>
-          <t>[redacted] JWT literal</t>
+          <t>[redacted] database password literal</t>
         </is>
       </c>
       <c r="V97" s="2" t="inlineStr">
         <is>
-          <t>SECRET-JWT-LITERAL</t>
+          <t>SECRET-DB-PASSWORD-LITERAL</t>
         </is>
       </c>
     </row>
@@ -9301,11 +9377,11 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>test/api/mocha/data/acl/directAcl.test.js</t>
+          <t>test/api/README.md</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
@@ -9319,14 +9395,14 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>JWT literal</t>
+          <t>Database password literal (MYSQL_ROOT_PASSWORD)</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr"/>
       <c r="H98" s="2" t="inlineStr"/>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>Embedded signed token (type: bearer token fixture)</t>
+          <t>Credential literal (type: database password)</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr"/>
@@ -9353,23 +9429,23 @@
       </c>
       <c r="P98" s="2" t="inlineStr"/>
       <c r="Q98" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R98" s="2" t="inlineStr">
         <is>
-          <t>Test fixture tokens; they are signed with test keys and expire.</t>
+          <t>Literal credential in test/CI configuration; must not be reused in production.</t>
         </is>
       </c>
       <c r="S98" s="2" t="inlineStr"/>
       <c r="T98" s="2" t="inlineStr"/>
       <c r="U98" s="2" t="inlineStr">
         <is>
-          <t>[redacted] JWT literal</t>
+          <t>[redacted] database password literal</t>
         </is>
       </c>
       <c r="V98" s="2" t="inlineStr">
         <is>
-          <t>SECRET-JWT-LITERAL</t>
+          <t>SECRET-DB-PASSWORD-LITERAL</t>
         </is>
       </c>
     </row>
@@ -9381,11 +9457,11 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>test/api/mocha/data/acl/groupAcl.test.js</t>
+          <t>test/api/README.md</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
@@ -9399,14 +9475,14 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>JWT literal</t>
+          <t>Database password literal (MYSQL_PASSWORD)</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr"/>
       <c r="H99" s="2" t="inlineStr"/>
       <c r="I99" s="2" t="inlineStr">
         <is>
-          <t>Embedded signed token (type: bearer token fixture)</t>
+          <t>Credential literal (type: database password)</t>
         </is>
       </c>
       <c r="J99" s="2" t="inlineStr"/>
@@ -9433,23 +9509,23 @@
       </c>
       <c r="P99" s="2" t="inlineStr"/>
       <c r="Q99" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R99" s="2" t="inlineStr">
         <is>
-          <t>Test fixture tokens; they are signed with test keys and expire.</t>
+          <t>Literal credential in test/CI configuration; must not be reused in production.</t>
         </is>
       </c>
       <c r="S99" s="2" t="inlineStr"/>
       <c r="T99" s="2" t="inlineStr"/>
       <c r="U99" s="2" t="inlineStr">
         <is>
-          <t>[redacted] JWT literal</t>
+          <t>[redacted] database password literal</t>
         </is>
       </c>
       <c r="V99" s="2" t="inlineStr">
         <is>
-          <t>SECRET-JWT-LITERAL</t>
+          <t>SECRET-DB-PASSWORD-LITERAL</t>
         </is>
       </c>
     </row>
@@ -9461,11 +9537,11 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>test/api/mocha/integration/access.test.js</t>
+          <t>test/api/mocha/cross-boundary/lvl1.test.js</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
@@ -9517,7 +9593,7 @@
       </c>
       <c r="R100" s="2" t="inlineStr">
         <is>
-          <t>Test fixture tokens; they are signed with test keys and expire. 3 occurrences in this file; first occurrence listed.</t>
+          <t>Test fixture tokens; they are signed with test keys and expire. 2 occurrences in this file; first occurrence listed.</t>
         </is>
       </c>
       <c r="S100" s="2" t="inlineStr"/>
@@ -9541,11 +9617,11 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>test/api/mocha/integration/aclResolution.test.js</t>
+          <t>test/api/mocha/data/acl/directAcl.test.js</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
@@ -9597,7 +9673,7 @@
       </c>
       <c r="R101" s="2" t="inlineStr">
         <is>
-          <t>Test fixture tokens; they are signed with test keys and expire. 2 occurrences in this file; first occurrence listed.</t>
+          <t>Test fixture tokens; they are signed with test keys and expire.</t>
         </is>
       </c>
       <c r="S101" s="2" t="inlineStr"/>
@@ -9621,11 +9697,11 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>test/api/mocha/integration/asset.test.js</t>
+          <t>test/api/mocha/data/acl/groupAcl.test.js</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
@@ -9701,11 +9777,11 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>test/api/mocha/integration/collection.test.js</t>
+          <t>test/api/mocha/integration/access.test.js</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
@@ -9781,7 +9857,7 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>test/api/mocha/integration/collectionTaskConfig.test.js</t>
+          <t>test/api/mocha/integration/aclResolution.test.js</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -9837,7 +9913,7 @@
       </c>
       <c r="R104" s="2" t="inlineStr">
         <is>
-          <t>Test fixture tokens; they are signed with test keys and expire. 3 occurrences in this file; first occurrence listed.</t>
+          <t>Test fixture tokens; they are signed with test keys and expire. 2 occurrences in this file; first occurrence listed.</t>
         </is>
       </c>
       <c r="S104" s="2" t="inlineStr"/>
@@ -9861,7 +9937,7 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>test/api/mocha/integration/deleteHandling.test.js</t>
+          <t>test/api/mocha/integration/asset.test.js</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -9941,11 +10017,11 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>test/api/mocha/integration/grantChange.test.js</t>
+          <t>test/api/mocha/integration/collection.test.js</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
@@ -9997,7 +10073,7 @@
       </c>
       <c r="R106" s="2" t="inlineStr">
         <is>
-          <t>Test fixture tokens; they are signed with test keys and expire.</t>
+          <t>Test fixture tokens; they are signed with test keys and expire. 3 occurrences in this file; first occurrence listed.</t>
         </is>
       </c>
       <c r="S106" s="2" t="inlineStr"/>
@@ -10021,11 +10097,11 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>test/api/mocha/integration/job.test.js</t>
+          <t>test/api/mocha/integration/collectionTaskConfig.test.js</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
@@ -10077,7 +10153,7 @@
       </c>
       <c r="R107" s="2" t="inlineStr">
         <is>
-          <t>Test fixture tokens; they are signed with test keys and expire.</t>
+          <t>Test fixture tokens; they are signed with test keys and expire. 3 occurrences in this file; first occurrence listed.</t>
         </is>
       </c>
       <c r="S107" s="2" t="inlineStr"/>
@@ -10101,11 +10177,11 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>test/api/mocha/integration/metrics.test.js</t>
+          <t>test/api/mocha/integration/deleteHandling.test.js</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
@@ -10181,11 +10257,11 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>test/api/mocha/integration/review.test.js</t>
+          <t>test/api/mocha/integration/grantChange.test.js</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
@@ -10261,11 +10337,11 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>test/api/mocha/integration/roleResolution.test.js</t>
+          <t>test/api/mocha/integration/job.test.js</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
@@ -10317,7 +10393,7 @@
       </c>
       <c r="R110" s="2" t="inlineStr">
         <is>
-          <t>Test fixture tokens; they are signed with test keys and expire. 2 occurrences in this file; first occurrence listed.</t>
+          <t>Test fixture tokens; they are signed with test keys and expire.</t>
         </is>
       </c>
       <c r="S110" s="2" t="inlineStr"/>
@@ -10341,11 +10417,11 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>test/api/mocha/integration/stig.test.js</t>
+          <t>test/api/mocha/integration/metrics.test.js</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
@@ -10421,11 +10497,11 @@
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>test/api/mocha/integration/userStatus.test.js</t>
+          <t>test/api/mocha/integration/review.test.js</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
@@ -10477,7 +10553,7 @@
       </c>
       <c r="R112" s="2" t="inlineStr">
         <is>
-          <t>Test fixture tokens; they are signed with test keys and expire. 2 occurrences in this file; first occurrence listed.</t>
+          <t>Test fixture tokens; they are signed with test keys and expire.</t>
         </is>
       </c>
       <c r="S112" s="2" t="inlineStr"/>
@@ -10501,11 +10577,11 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>test/api/mocha/iterations.js</t>
+          <t>test/api/mocha/integration/roleResolution.test.js</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
@@ -10557,7 +10633,7 @@
       </c>
       <c r="R113" s="2" t="inlineStr">
         <is>
-          <t>Test fixture tokens; they are signed with test keys and expire. 6 occurrences in this file; first occurrence listed.</t>
+          <t>Test fixture tokens; they are signed with test keys and expire. 2 occurrences in this file; first occurrence listed.</t>
         </is>
       </c>
       <c r="S113" s="2" t="inlineStr"/>
@@ -10581,11 +10657,11 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>test/api/mocha/security/reviewCrossCollectionWrite.test.js</t>
+          <t>test/api/mocha/integration/stig.test.js</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
-        <v>71</v>
+        <v>15</v>
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
@@ -10637,7 +10713,7 @@
       </c>
       <c r="R114" s="2" t="inlineStr">
         <is>
-          <t>Test fixture tokens; they are signed with test keys and expire. 2 occurrences in this file; first occurrence listed.</t>
+          <t>Test fixture tokens; they are signed with test keys and expire.</t>
         </is>
       </c>
       <c r="S114" s="2" t="inlineStr"/>
@@ -10661,11 +10737,11 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>test/api/mocha/testConfig.js</t>
+          <t>test/api/mocha/integration/userStatus.test.js</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
@@ -10717,7 +10793,7 @@
       </c>
       <c r="R115" s="2" t="inlineStr">
         <is>
-          <t>Test fixture tokens; they are signed with test keys and expire.</t>
+          <t>Test fixture tokens; they are signed with test keys and expire. 2 occurrences in this file; first occurrence listed.</t>
         </is>
       </c>
       <c r="S115" s="2" t="inlineStr"/>
@@ -10741,11 +10817,11 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>test/api/runMocha.sh</t>
+          <t>test/api/mocha/iterations.js</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
-        <v>112</v>
+        <v>8</v>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
@@ -10759,14 +10835,14 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>Database password literal (STIGMAN_DB_PASSWORD)</t>
+          <t>JWT literal</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr"/>
       <c r="H116" s="2" t="inlineStr"/>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>Credential literal (type: database password)</t>
+          <t>Embedded signed token (type: bearer token fixture)</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr"/>
@@ -10793,23 +10869,23 @@
       </c>
       <c r="P116" s="2" t="inlineStr"/>
       <c r="Q116" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R116" s="2" t="inlineStr">
         <is>
-          <t>Literal credential in test/CI configuration; must not be reused in production.</t>
+          <t>Test fixture tokens; they are signed with test keys and expire. 6 occurrences in this file; first occurrence listed.</t>
         </is>
       </c>
       <c r="S116" s="2" t="inlineStr"/>
       <c r="T116" s="2" t="inlineStr"/>
       <c r="U116" s="2" t="inlineStr">
         <is>
-          <t>[redacted] database password literal</t>
+          <t>[redacted] JWT literal</t>
         </is>
       </c>
       <c r="V116" s="2" t="inlineStr">
         <is>
-          <t>SECRET-DB-PASSWORD-LITERAL</t>
+          <t>SECRET-JWT-LITERAL</t>
         </is>
       </c>
     </row>
@@ -10821,11 +10897,11 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>test/state/mocha/bootstrap.test.js</t>
+          <t>test/api/mocha/security/reviewCrossCollectionWrite.test.js</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
-        <v>108</v>
+        <v>71</v>
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
@@ -10839,14 +10915,14 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>Database password literal (STIGMAN_DB_PASSWORD)</t>
+          <t>JWT literal</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr"/>
       <c r="H117" s="2" t="inlineStr"/>
       <c r="I117" s="2" t="inlineStr">
         <is>
-          <t>Credential literal (type: database password)</t>
+          <t>Embedded signed token (type: bearer token fixture)</t>
         </is>
       </c>
       <c r="J117" s="2" t="inlineStr"/>
@@ -10873,23 +10949,23 @@
       </c>
       <c r="P117" s="2" t="inlineStr"/>
       <c r="Q117" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R117" s="2" t="inlineStr">
         <is>
-          <t>Literal credential in test/CI configuration; must not be reused in production.</t>
+          <t>Test fixture tokens; they are signed with test keys and expire. 2 occurrences in this file; first occurrence listed.</t>
         </is>
       </c>
       <c r="S117" s="2" t="inlineStr"/>
       <c r="T117" s="2" t="inlineStr"/>
       <c r="U117" s="2" t="inlineStr">
         <is>
-          <t>[redacted] database password literal</t>
+          <t>[redacted] JWT literal</t>
         </is>
       </c>
       <c r="V117" s="2" t="inlineStr">
         <is>
-          <t>SECRET-DB-PASSWORD-LITERAL</t>
+          <t>SECRET-JWT-LITERAL</t>
         </is>
       </c>
     </row>
@@ -10901,11 +10977,11 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>test/state/mocha/bootstrap.test.js</t>
+          <t>test/api/mocha/testConfig.js</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
-        <v>186</v>
+        <v>3</v>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
@@ -10919,14 +10995,14 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>Database password literal (STIGMAN_DB_PASSWORD)</t>
+          <t>JWT literal</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr"/>
       <c r="H118" s="2" t="inlineStr"/>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>Credential literal (type: database password)</t>
+          <t>Embedded signed token (type: bearer token fixture)</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr"/>
@@ -10953,23 +11029,23 @@
       </c>
       <c r="P118" s="2" t="inlineStr"/>
       <c r="Q118" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R118" s="2" t="inlineStr">
         <is>
-          <t>Literal credential in test/CI configuration; must not be reused in production.</t>
+          <t>Test fixture tokens; they are signed with test keys and expire.</t>
         </is>
       </c>
       <c r="S118" s="2" t="inlineStr"/>
       <c r="T118" s="2" t="inlineStr"/>
       <c r="U118" s="2" t="inlineStr">
         <is>
-          <t>[redacted] database password literal</t>
+          <t>[redacted] JWT literal</t>
         </is>
       </c>
       <c r="V118" s="2" t="inlineStr">
         <is>
-          <t>SECRET-DB-PASSWORD-LITERAL</t>
+          <t>SECRET-JWT-LITERAL</t>
         </is>
       </c>
     </row>
@@ -10981,11 +11057,11 @@
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>test/state/mocha/bootstrap.test.js</t>
+          <t>test/api/runMocha.sh</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
-        <v>246</v>
+        <v>112</v>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
@@ -11065,7 +11141,7 @@
         </is>
       </c>
       <c r="C120" s="2" t="n">
-        <v>310</v>
+        <v>108</v>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
@@ -11145,7 +11221,7 @@
         </is>
       </c>
       <c r="C121" s="2" t="n">
-        <v>383</v>
+        <v>186</v>
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
@@ -11225,7 +11301,7 @@
         </is>
       </c>
       <c r="C122" s="2" t="n">
-        <v>407</v>
+        <v>246</v>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
@@ -11305,7 +11381,7 @@
         </is>
       </c>
       <c r="C123" s="2" t="n">
-        <v>431</v>
+        <v>310</v>
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
@@ -11381,11 +11457,11 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>test/state/mocha/db.test.js</t>
+          <t>test/state/mocha/bootstrap.test.js</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
-        <v>30</v>
+        <v>383</v>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
@@ -11461,11 +11537,11 @@
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>test/state/mocha/db.test.js</t>
+          <t>test/state/mocha/bootstrap.test.js</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
-        <v>127</v>
+        <v>407</v>
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
@@ -11541,11 +11617,11 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>test/state/mocha/jwks.test.js</t>
+          <t>test/state/mocha/bootstrap.test.js</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
-        <v>37</v>
+        <v>431</v>
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
@@ -11621,11 +11697,11 @@
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>test/state/mocha/lib.js</t>
+          <t>test/state/mocha/db.test.js</t>
         </is>
       </c>
       <c r="C127" s="2" t="n">
-        <v>236</v>
+        <v>30</v>
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
@@ -11639,7 +11715,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>Database password literal (MYSQL_ROOT_PASSWORD)</t>
+          <t>Database password literal (STIGMAN_DB_PASSWORD)</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr"/>
@@ -11701,11 +11777,11 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>test/state/mocha/lib.js</t>
+          <t>test/state/mocha/db.test.js</t>
         </is>
       </c>
       <c r="C128" s="2" t="n">
-        <v>239</v>
+        <v>127</v>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
@@ -11719,7 +11795,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>Database password literal (MYSQL_PASSWORD)</t>
+          <t>Database password literal (STIGMAN_DB_PASSWORD)</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr"/>
@@ -11781,11 +11857,11 @@
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>test/state/mocha/oidc.test.js</t>
+          <t>test/state/mocha/jwks.test.js</t>
         </is>
       </c>
       <c r="C129" s="2" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
@@ -11861,11 +11937,11 @@
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>test/state/mocha/tokenValidation.test.js</t>
+          <t>test/state/mocha/lib.js</t>
         </is>
       </c>
       <c r="C130" s="2" t="n">
-        <v>32</v>
+        <v>236</v>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
@@ -11879,7 +11955,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>Database password literal (STIGMAN_DB_PASSWORD)</t>
+          <t>Database password literal (MYSQL_ROOT_PASSWORD)</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr"/>
@@ -11941,11 +12017,11 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>test/state/mocha/tokenValidation.test.js</t>
+          <t>test/state/mocha/lib.js</t>
         </is>
       </c>
       <c r="C131" s="2" t="n">
-        <v>132</v>
+        <v>239</v>
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
@@ -11959,7 +12035,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>Database password literal (STIGMAN_DB_PASSWORD)</t>
+          <t>Database password literal (MYSQL_PASSWORD)</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr"/>
@@ -12021,11 +12097,11 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>test/utils/appdata-update.js</t>
+          <t>test/state/mocha/oidc.test.js</t>
         </is>
       </c>
       <c r="C132" s="2" t="n">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
@@ -12039,14 +12115,14 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>JWT literal</t>
+          <t>Database password literal (STIGMAN_DB_PASSWORD)</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr"/>
       <c r="H132" s="2" t="inlineStr"/>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>Embedded signed token (type: bearer token fixture)</t>
+          <t>Credential literal (type: database password)</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr"/>
@@ -12073,23 +12149,23 @@
       </c>
       <c r="P132" s="2" t="inlineStr"/>
       <c r="Q132" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R132" s="2" t="inlineStr">
         <is>
-          <t>Test fixture tokens; they are signed with test keys and expire.</t>
+          <t>Literal credential in test/CI configuration; must not be reused in production.</t>
         </is>
       </c>
       <c r="S132" s="2" t="inlineStr"/>
       <c r="T132" s="2" t="inlineStr"/>
       <c r="U132" s="2" t="inlineStr">
         <is>
-          <t>[redacted] JWT literal</t>
+          <t>[redacted] database password literal</t>
         </is>
       </c>
       <c r="V132" s="2" t="inlineStr">
         <is>
-          <t>SECRET-JWT-LITERAL</t>
+          <t>SECRET-DB-PASSWORD-LITERAL</t>
         </is>
       </c>
     </row>
@@ -12101,11 +12177,11 @@
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>test/utils/mockOidc.js</t>
+          <t>test/state/mocha/tokenValidation.test.js</t>
         </is>
       </c>
       <c r="C133" s="2" t="n">
-        <v>53</v>
+        <v>32</v>
       </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
@@ -12119,14 +12195,14 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>Private key (JWK private exponent)</t>
+          <t>Database password literal (STIGMAN_DB_PASSWORD)</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr"/>
       <c r="H133" s="2" t="inlineStr"/>
       <c r="I133" s="2" t="inlineStr">
         <is>
-          <t>Embedded RSA private key component (type: JWK private key)</t>
+          <t>Credential literal (type: database password)</t>
         </is>
       </c>
       <c r="J133" s="2" t="inlineStr"/>
@@ -12138,12 +12214,12 @@
       </c>
       <c r="M133" s="2" t="inlineStr">
         <is>
-          <t>Quantum-vulnerable (Shor)</t>
+          <t>Not applicable (no quantum-relevant primitive)</t>
         </is>
       </c>
       <c r="N133" s="2" t="inlineStr">
         <is>
-          <t>ML-DSA-87 (FIPS 204) or SLH-DSA (FIPS 205) for signatures</t>
+          <t>None required</t>
         </is>
       </c>
       <c r="O133" s="2" t="inlineStr">
@@ -12157,19 +12233,19 @@
       </c>
       <c r="R133" s="2" t="inlineStr">
         <is>
-          <t>Reproduces a public, known-insecure IdP key for negative tests; the kid is on the application denylist.</t>
+          <t>Literal credential in test/CI configuration; must not be reused in production.</t>
         </is>
       </c>
       <c r="S133" s="2" t="inlineStr"/>
       <c r="T133" s="2" t="inlineStr"/>
       <c r="U133" s="2" t="inlineStr">
         <is>
-          <t>[redacted] JWK private component</t>
+          <t>[redacted] database password literal</t>
         </is>
       </c>
       <c r="V133" s="2" t="inlineStr">
         <is>
-          <t>SECRET-JWK-PRIVATE</t>
+          <t>SECRET-DB-PASSWORD-LITERAL</t>
         </is>
       </c>
     </row>
@@ -12181,39 +12257,35 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/api-audit-test-coverage-response.yml</t>
+          <t>test/state/mocha/tokenValidation.test.js</t>
         </is>
       </c>
       <c r="C134" s="2" t="n">
-        <v>171</v>
+        <v>132</v>
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>Secret reference</t>
+          <t>Secret</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>CI secret reference (GITHUB_TOKEN)</t>
+          <t>Database password literal (STIGMAN_DB_PASSWORD)</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr"/>
       <c r="H134" s="2" t="inlineStr"/>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>Secret injected by the CI secret store (not stored in repository)</t>
-        </is>
-      </c>
-      <c r="J134" s="2" t="inlineStr">
-        <is>
-          <t>GitHub Actions</t>
-        </is>
-      </c>
+          <t>Credential literal (type: database password)</t>
+        </is>
+      </c>
+      <c r="J134" s="2" t="inlineStr"/>
       <c r="K134" s="2" t="inlineStr"/>
       <c r="L134" s="2" t="inlineStr">
         <is>
@@ -12232,28 +12304,28 @@
       </c>
       <c r="O134" s="2" t="inlineStr">
         <is>
-          <t>Configurable</t>
+          <t>Hardcoded</t>
         </is>
       </c>
       <c r="P134" s="2" t="inlineStr"/>
       <c r="Q134" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R134" s="2" t="inlineStr">
         <is>
-          <t>Reference only; value held by the CI platform.</t>
+          <t>Literal credential in test/CI configuration; must not be reused in production.</t>
         </is>
       </c>
       <c r="S134" s="2" t="inlineStr"/>
       <c r="T134" s="2" t="inlineStr"/>
       <c r="U134" s="2" t="inlineStr">
         <is>
-          <t>${{ secrets.GITHUB_TOKEN }}</t>
+          <t>[redacted] database password literal</t>
         </is>
       </c>
       <c r="V134" s="2" t="inlineStr">
         <is>
-          <t>SECRET-CI-REFERENCE</t>
+          <t>SECRET-DB-PASSWORD-LITERAL</t>
         </is>
       </c>
     </row>
@@ -12265,39 +12337,35 @@
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/api-audit-test-coverage-response.yml</t>
+          <t>test/utils/appdata-update.js</t>
         </is>
       </c>
       <c r="C135" s="2" t="n">
-        <v>172</v>
+        <v>7</v>
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>Secret reference</t>
+          <t>Secret</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>CI secret reference (SONAR_TOKEN_API)</t>
+          <t>JWT literal</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr"/>
       <c r="H135" s="2" t="inlineStr"/>
       <c r="I135" s="2" t="inlineStr">
         <is>
-          <t>Secret injected by the CI secret store (not stored in repository)</t>
-        </is>
-      </c>
-      <c r="J135" s="2" t="inlineStr">
-        <is>
-          <t>GitHub Actions</t>
-        </is>
-      </c>
+          <t>Embedded signed token (type: bearer token fixture)</t>
+        </is>
+      </c>
+      <c r="J135" s="2" t="inlineStr"/>
       <c r="K135" s="2" t="inlineStr"/>
       <c r="L135" s="2" t="inlineStr">
         <is>
@@ -12316,7 +12384,7 @@
       </c>
       <c r="O135" s="2" t="inlineStr">
         <is>
-          <t>Configurable</t>
+          <t>Hardcoded</t>
         </is>
       </c>
       <c r="P135" s="2" t="inlineStr"/>
@@ -12325,19 +12393,19 @@
       </c>
       <c r="R135" s="2" t="inlineStr">
         <is>
-          <t>Reference only; value held by the CI platform.</t>
+          <t>Test fixture tokens; they are signed with test keys and expire.</t>
         </is>
       </c>
       <c r="S135" s="2" t="inlineStr"/>
       <c r="T135" s="2" t="inlineStr"/>
       <c r="U135" s="2" t="inlineStr">
         <is>
-          <t>${{ secrets.SONAR_TOKEN_API }}</t>
+          <t>[redacted] JWT literal</t>
         </is>
       </c>
       <c r="V135" s="2" t="inlineStr">
         <is>
-          <t>SECRET-CI-REFERENCE</t>
+          <t>SECRET-JWT-LITERAL</t>
         </is>
       </c>
     </row>
@@ -12349,39 +12417,35 @@
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/build-binary-artifacts.yml</t>
+          <t>test/utils/mockOidc.js</t>
         </is>
       </c>
       <c r="C136" s="2" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>Secret reference</t>
+          <t>Secret</t>
         </is>
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>CI secret reference (STIGMAN_PRIVATE_KEY)</t>
+          <t>Private key (JWK private exponent)</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr"/>
       <c r="H136" s="2" t="inlineStr"/>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>Secret injected by the CI secret store (not stored in repository)</t>
-        </is>
-      </c>
-      <c r="J136" s="2" t="inlineStr">
-        <is>
-          <t>GitHub Actions</t>
-        </is>
-      </c>
+          <t>Embedded RSA private key component (type: JWK private key)</t>
+        </is>
+      </c>
+      <c r="J136" s="2" t="inlineStr"/>
       <c r="K136" s="2" t="inlineStr"/>
       <c r="L136" s="2" t="inlineStr">
         <is>
@@ -12390,38 +12454,38 @@
       </c>
       <c r="M136" s="2" t="inlineStr">
         <is>
-          <t>Not applicable (no quantum-relevant primitive)</t>
+          <t>Quantum-vulnerable (Shor)</t>
         </is>
       </c>
       <c r="N136" s="2" t="inlineStr">
         <is>
-          <t>None required</t>
+          <t>ML-DSA-87 (FIPS 204) or SLH-DSA (FIPS 205) for signatures</t>
         </is>
       </c>
       <c r="O136" s="2" t="inlineStr">
         <is>
-          <t>Configurable</t>
+          <t>Hardcoded</t>
         </is>
       </c>
       <c r="P136" s="2" t="inlineStr"/>
       <c r="Q136" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R136" s="2" t="inlineStr">
         <is>
-          <t>Reference only; value held by the CI platform.</t>
+          <t>Reproduces a public, known-insecure IdP key for negative tests; the kid is on the application denylist.</t>
         </is>
       </c>
       <c r="S136" s="2" t="inlineStr"/>
       <c r="T136" s="2" t="inlineStr"/>
       <c r="U136" s="2" t="inlineStr">
         <is>
-          <t>${{ secrets.STIGMAN_PRIVATE_KEY }}</t>
+          <t>[redacted] JWK private component</t>
         </is>
       </c>
       <c r="V136" s="2" t="inlineStr">
         <is>
-          <t>SECRET-CI-REFERENCE</t>
+          <t>SECRET-JWK-PRIVATE</t>
         </is>
       </c>
     </row>
@@ -12433,11 +12497,11 @@
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/client-sonarcloud.yml</t>
+          <t>.github/workflows/api-audit-test-coverage-response.yml</t>
         </is>
       </c>
       <c r="C137" s="2" t="n">
-        <v>48</v>
+        <v>171</v>
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
@@ -12517,11 +12581,11 @@
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/client-sonarcloud.yml</t>
+          <t>.github/workflows/api-audit-test-coverage-response.yml</t>
         </is>
       </c>
       <c r="C138" s="2" t="n">
-        <v>49</v>
+        <v>172</v>
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
@@ -12535,7 +12599,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>CI secret reference (SONAR_TOKEN_CLIENT)</t>
+          <t>CI secret reference (SONAR_TOKEN_API)</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr"/>
@@ -12584,7 +12648,7 @@
       <c r="T138" s="2" t="inlineStr"/>
       <c r="U138" s="2" t="inlineStr">
         <is>
-          <t>${{ secrets.SONAR_TOKEN_CLIENT }}</t>
+          <t>${{ secrets.SONAR_TOKEN_API }}</t>
         </is>
       </c>
       <c r="V138" s="2" t="inlineStr">
@@ -12601,11 +12665,11 @@
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/pub-docker.yml</t>
+          <t>.github/workflows/build-binary-artifacts.yml</t>
         </is>
       </c>
       <c r="C139" s="2" t="n">
-        <v>77</v>
+        <v>49</v>
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
@@ -12619,7 +12683,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>CI secret reference (DOCKERHUB_ORG_OWNER_USERNAME)</t>
+          <t>CI secret reference (STIGMAN_PRIVATE_KEY)</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr"/>
@@ -12668,7 +12732,7 @@
       <c r="T139" s="2" t="inlineStr"/>
       <c r="U139" s="2" t="inlineStr">
         <is>
-          <t>${{ secrets.DOCKERHUB_ORG_OWNER_USERNAME }}</t>
+          <t>${{ secrets.STIGMAN_PRIVATE_KEY }}</t>
         </is>
       </c>
       <c r="V139" s="2" t="inlineStr">
@@ -12685,11 +12749,11 @@
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/pub-docker.yml</t>
+          <t>.github/workflows/client-sonarcloud.yml</t>
         </is>
       </c>
       <c r="C140" s="2" t="n">
-        <v>78</v>
+        <v>48</v>
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
@@ -12703,7 +12767,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>CI secret reference (DOCKERHUB_ORG_OWNER_PW)</t>
+          <t>CI secret reference (GITHUB_TOKEN)</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr"/>
@@ -12752,7 +12816,7 @@
       <c r="T140" s="2" t="inlineStr"/>
       <c r="U140" s="2" t="inlineStr">
         <is>
-          <t>${{ secrets.DOCKERHUB_ORG_OWNER_PW }}</t>
+          <t>${{ secrets.GITHUB_TOKEN }}</t>
         </is>
       </c>
       <c r="V140" s="2" t="inlineStr">
@@ -12769,11 +12833,11 @@
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/pub-docker.yml</t>
+          <t>.github/workflows/client-sonarcloud.yml</t>
         </is>
       </c>
       <c r="C141" s="2" t="n">
-        <v>108</v>
+        <v>49</v>
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
@@ -12787,7 +12851,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>CI secret reference (DOCKERHUB_ORG_OWNER_USERNAME)</t>
+          <t>CI secret reference (SONAR_TOKEN_CLIENT)</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr"/>
@@ -12836,7 +12900,7 @@
       <c r="T141" s="2" t="inlineStr"/>
       <c r="U141" s="2" t="inlineStr">
         <is>
-          <t>${{ secrets.DOCKERHUB_ORG_OWNER_USERNAME }}</t>
+          <t>${{ secrets.SONAR_TOKEN_CLIENT }}</t>
         </is>
       </c>
       <c r="V141" s="2" t="inlineStr">
@@ -12857,7 +12921,7 @@
         </is>
       </c>
       <c r="C142" s="2" t="n">
-        <v>109</v>
+        <v>77</v>
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
@@ -12871,7 +12935,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>CI secret reference (DOCKERHUB_ORG_OWNER_PW)</t>
+          <t>CI secret reference (DOCKERHUB_ORG_OWNER_USERNAME)</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr"/>
@@ -12920,17 +12984,269 @@
       <c r="T142" s="2" t="inlineStr"/>
       <c r="U142" s="2" t="inlineStr">
         <is>
+          <t>${{ secrets.DOCKERHUB_ORG_OWNER_USERNAME }}</t>
+        </is>
+      </c>
+      <c r="V142" s="2" t="inlineStr">
+        <is>
+          <t>SECRET-CI-REFERENCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>CI-0142</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>.github/workflows/pub-docker.yml</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>Secret reference</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>CI secret reference (DOCKERHUB_ORG_OWNER_PW)</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="inlineStr"/>
+      <c r="H143" s="2" t="inlineStr"/>
+      <c r="I143" s="2" t="inlineStr">
+        <is>
+          <t>Secret injected by the CI secret store (not stored in repository)</t>
+        </is>
+      </c>
+      <c r="J143" s="2" t="inlineStr">
+        <is>
+          <t>GitHub Actions</t>
+        </is>
+      </c>
+      <c r="K143" s="2" t="inlineStr"/>
+      <c r="L143" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M143" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable (no quantum-relevant primitive)</t>
+        </is>
+      </c>
+      <c r="N143" s="2" t="inlineStr">
+        <is>
+          <t>None required</t>
+        </is>
+      </c>
+      <c r="O143" s="2" t="inlineStr">
+        <is>
+          <t>Configurable</t>
+        </is>
+      </c>
+      <c r="P143" s="2" t="inlineStr"/>
+      <c r="Q143" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="R143" s="2" t="inlineStr">
+        <is>
+          <t>Reference only; value held by the CI platform.</t>
+        </is>
+      </c>
+      <c r="S143" s="2" t="inlineStr"/>
+      <c r="T143" s="2" t="inlineStr"/>
+      <c r="U143" s="2" t="inlineStr">
+        <is>
           <t>${{ secrets.DOCKERHUB_ORG_OWNER_PW }}</t>
         </is>
       </c>
-      <c r="V142" s="2" t="inlineStr">
+      <c r="V143" s="2" t="inlineStr">
         <is>
           <t>SECRET-CI-REFERENCE</t>
         </is>
       </c>
     </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>CI-0143</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>.github/workflows/pub-docker.yml</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="n">
+        <v>108</v>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>Secret reference</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>CI secret reference (DOCKERHUB_ORG_OWNER_USERNAME)</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr"/>
+      <c r="H144" s="2" t="inlineStr"/>
+      <c r="I144" s="2" t="inlineStr">
+        <is>
+          <t>Secret injected by the CI secret store (not stored in repository)</t>
+        </is>
+      </c>
+      <c r="J144" s="2" t="inlineStr">
+        <is>
+          <t>GitHub Actions</t>
+        </is>
+      </c>
+      <c r="K144" s="2" t="inlineStr"/>
+      <c r="L144" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M144" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable (no quantum-relevant primitive)</t>
+        </is>
+      </c>
+      <c r="N144" s="2" t="inlineStr">
+        <is>
+          <t>None required</t>
+        </is>
+      </c>
+      <c r="O144" s="2" t="inlineStr">
+        <is>
+          <t>Configurable</t>
+        </is>
+      </c>
+      <c r="P144" s="2" t="inlineStr"/>
+      <c r="Q144" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="R144" s="2" t="inlineStr">
+        <is>
+          <t>Reference only; value held by the CI platform.</t>
+        </is>
+      </c>
+      <c r="S144" s="2" t="inlineStr"/>
+      <c r="T144" s="2" t="inlineStr"/>
+      <c r="U144" s="2" t="inlineStr">
+        <is>
+          <t>${{ secrets.DOCKERHUB_ORG_OWNER_USERNAME }}</t>
+        </is>
+      </c>
+      <c r="V144" s="2" t="inlineStr">
+        <is>
+          <t>SECRET-CI-REFERENCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>CI-0144</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>.github/workflows/pub-docker.yml</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="n">
+        <v>109</v>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>Secret reference</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>CI secret reference (DOCKERHUB_ORG_OWNER_PW)</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="inlineStr"/>
+      <c r="H145" s="2" t="inlineStr"/>
+      <c r="I145" s="2" t="inlineStr">
+        <is>
+          <t>Secret injected by the CI secret store (not stored in repository)</t>
+        </is>
+      </c>
+      <c r="J145" s="2" t="inlineStr">
+        <is>
+          <t>GitHub Actions</t>
+        </is>
+      </c>
+      <c r="K145" s="2" t="inlineStr"/>
+      <c r="L145" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M145" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable (no quantum-relevant primitive)</t>
+        </is>
+      </c>
+      <c r="N145" s="2" t="inlineStr">
+        <is>
+          <t>None required</t>
+        </is>
+      </c>
+      <c r="O145" s="2" t="inlineStr">
+        <is>
+          <t>Configurable</t>
+        </is>
+      </c>
+      <c r="P145" s="2" t="inlineStr"/>
+      <c r="Q145" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="R145" s="2" t="inlineStr">
+        <is>
+          <t>Reference only; value held by the CI platform.</t>
+        </is>
+      </c>
+      <c r="S145" s="2" t="inlineStr"/>
+      <c r="T145" s="2" t="inlineStr"/>
+      <c r="U145" s="2" t="inlineStr">
+        <is>
+          <t>${{ secrets.DOCKERHUB_ORG_OWNER_PW }}</t>
+        </is>
+      </c>
+      <c r="V145" s="2" t="inlineStr">
+        <is>
+          <t>SECRET-CI-REFERENCE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:V142">
+  <conditionalFormatting sqref="A2:V145">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
       <formula>$M2="Quantum-vulnerable (Shor)"</formula>
     </cfRule>
@@ -15889,7 +16205,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>CI-0056</t>
+          <t>CI-0056, CI-0057, CI-0058, CI-0059</t>
         </is>
       </c>
     </row>
@@ -15926,7 +16242,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>CI-0061</t>
+          <t>CI-0064</t>
         </is>
       </c>
     </row>
@@ -15959,7 +16275,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>CI-0070</t>
+          <t>CI-0073</t>
         </is>
       </c>
     </row>
@@ -15977,7 +16293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16312,6 +16628,126 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>CI-0057</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>root.json</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>ECDSA (X.509 certificate)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Hardcoded</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Trust root keys are static ECDSA public keys embedded in root.json.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Track registry/Notary support for PQC signatures; re-issue trust roots when available.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>CI-0058</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>root.json</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>ECDSA</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Hardcoded</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Trust root keys are static ECDSA public keys embedded in root.json.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Track registry/Notary support for PQC signatures; re-issue trust roots when available.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>CI-0059</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>root.json</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>ECDSA</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Hardcoded</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Trust root keys are static ECDSA public keys embedded in root.json.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Track registry/Notary support for PQC signatures; re-issue trust roots when available.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -16326,7 +16762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17100,7 +17536,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>CI-0070</t>
+          <t>CI-0057</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -17108,11 +17544,11 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Dockerfile</t>
+          <t>root.json</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
@@ -17121,52 +17557,52 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Node.js/OpenSSL runtime (container base image)</t>
+          <t>ECDSA (X.509 certificate)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Protocol/configuration — inherits class of negotiated algorithms</t>
+          <t>Quantum-vulnerable (Shor)</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>TLS 1.3 with ML-KEM key establishment and ML-DSA certificates when available</t>
+          <t>ML-DSA (FIPS 204) or LMS/XMSS (SP 800-208) for software signing</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Upstream Node.js image publisher (mutable tag)</t>
+          <t>Container registry Notary service and consumer docker clients</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Pin a specific Node.js LTS major (24.x) with OpenSSL 3.5+ and record it in the inventory on each release.</t>
+          <t>Track registry/Notary support for PQC signatures; re-issue trust roots when available.</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Phase 0 / Phase 1</t>
+          <t>Phase 3</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Tag is mutable; the OpenSSL version that decides ML-KEM/ML-DSA availability is not pinned.</t>
+          <t>Image signature trust roots are ECDSA; verification keys are pinned in this file.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>CI-0009</t>
+          <t>CI-0058</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>test/api/mock-keycloak-test-cases/no-jwks/auth/realms/stigman/protocol/openid-connect/certs</t>
+          <t>root.json</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
@@ -17174,28 +17610,32 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Repository</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>RSA (JWK), alg=RS256</t>
+          <t>ECDSA</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Deprecated/weak regardless of PQC</t>
+          <t>Quantum-vulnerable (Shor)</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>ML-DSA-87 (FIPS 204) or SLH-DSA (FIPS 205) for signatures</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr"/>
+          <t>ML-DSA (FIPS 204) or LMS/XMSS (SP 800-208) for software signing</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Container registry Notary service and consumer docker clients</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Track; no change until dependency supports PQC.</t>
+          <t>Track registry/Notary support for PQC signatures; re-issue trust roots when available.</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -17205,22 +17645,22 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>RSA-1024 is below the SP 800-131A Rev. 2 floor. Static test JWKS; the key is the widely published insecure default and is on the application denylist. Test scope: not deployed.</t>
+          <t>Image signature trust roots are ECDSA; verification keys are pinned in this file.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>CI-0010</t>
+          <t>CI-0059</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>test/api/mock-keycloak-test-cases/secure-kid/auth/realms/stigman/protocol/openid-connect/certs</t>
+          <t>root.json</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
@@ -17228,28 +17668,32 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Repository</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>RSA (JWK), alg=RS256</t>
+          <t>ECDSA</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Deprecated/weak regardless of PQC</t>
+          <t>Quantum-vulnerable (Shor)</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>ML-DSA-87 (FIPS 204) or SLH-DSA (FIPS 205) for signatures</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr"/>
+          <t>ML-DSA (FIPS 204) or LMS/XMSS (SP 800-208) for software signing</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Container registry Notary service and consumer docker clients</t>
+        </is>
+      </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Track; no change until dependency supports PQC.</t>
+          <t>Track registry/Notary support for PQC signatures; re-issue trust roots when available.</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -17259,68 +17703,72 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>RSA-1024 is below the SP 800-131A Rev. 2 floor. Static test JWKS; the key is the widely published insecure default and is on the application denylist. Test scope: not deployed.</t>
+          <t>Image signature trust roots are ECDSA; verification keys are pinned in this file.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>CI-0011</t>
+          <t>CI-0073</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>test/api/mock-keycloak/auth/realms/stigman/protocol/openid-connect/certs</t>
+          <t>Dockerfile</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Repository</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>RSA (JWK), alg=RS256</t>
+          <t>Node.js/OpenSSL runtime (container base image)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Deprecated/weak regardless of PQC</t>
+          <t>Protocol/configuration — inherits class of negotiated algorithms</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>ML-DSA-87 (FIPS 204) or SLH-DSA (FIPS 205) for signatures</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr"/>
+          <t>TLS 1.3 with ML-KEM key establishment and ML-DSA certificates when available</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Upstream Node.js image publisher (mutable tag)</t>
+        </is>
+      </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Track; no change until dependency supports PQC.</t>
+          <t>Pin a specific Node.js LTS major (24.x) with OpenSSL 3.5+ and record it in the inventory on each release.</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Phase 3</t>
+          <t>Phase 0 / Phase 1</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>RSA-1024 is below the SP 800-131A Rev. 2 floor. Static test JWKS; the key is the widely published insecure default and is on the application denylist. Test scope: not deployed.</t>
+          <t>Tag is mutable; the OpenSSL version that decides ML-KEM/ML-DSA availability is not pinned.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>CI-0017</t>
+          <t>CI-0009</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -17328,11 +17776,11 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>test/utils/mockOidc.js</t>
+          <t>test/api/mock-keycloak-test-cases/no-jwks/auth/realms/stigman/protocol/openid-connect/certs</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
@@ -17341,7 +17789,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>RSA</t>
+          <t>RSA (JWK), alg=RS256</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -17357,7 +17805,7 @@
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Replace with configurable key type/size; add ML-DSA option when jsonwebtoken or a successor library supports it.</t>
+          <t>Track; no change until dependency supports PQC.</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -17367,14 +17815,14 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>RSA-1024 is below the 2048-bit floor of SP 800-131A Rev. 2 and is quantum-vulnerable. Generates the signing key pair used to issue tokens; algorithm and size are literals in code. Test scope: not deployed.</t>
+          <t>RSA-1024 is below the SP 800-131A Rev. 2 floor. Static test JWKS; the key is the widely published insecure default and is on the application denylist. Test scope: not deployed.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>CI-0018</t>
+          <t>CI-0010</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
@@ -17382,11 +17830,11 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>test/utils/mockOidc.js</t>
+          <t>test/api/mock-keycloak-test-cases/secure-kid/auth/realms/stigman/protocol/openid-connect/certs</t>
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
@@ -17395,7 +17843,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>RSA</t>
+          <t>RSA (JWK), alg=RS256</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -17411,15 +17859,177 @@
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr">
         <is>
+          <t>Track; no change until dependency supports PQC.</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>RSA-1024 is below the SP 800-131A Rev. 2 floor. Static test JWKS; the key is the widely published insecure default and is on the application denylist. Test scope: not deployed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>CI-0011</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>test/api/mock-keycloak/auth/realms/stigman/protocol/openid-connect/certs</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>RSA (JWK), alg=RS256</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Deprecated/weak regardless of PQC</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>ML-DSA-87 (FIPS 204) or SLH-DSA (FIPS 205) for signatures</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Track; no change until dependency supports PQC.</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>RSA-1024 is below the SP 800-131A Rev. 2 floor. Static test JWKS; the key is the widely published insecure default and is on the application denylist. Test scope: not deployed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>CI-0017</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>test/utils/mockOidc.js</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>RSA</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Deprecated/weak regardless of PQC</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>ML-DSA-87 (FIPS 204) or SLH-DSA (FIPS 205) for signatures</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Replace with configurable key type/size; add ML-DSA option when jsonwebtoken or a successor library supports it.</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>RSA-1024 is below the 2048-bit floor of SP 800-131A Rev. 2 and is quantum-vulnerable. Generates the signing key pair used to issue tokens; algorithm and size are literals in code. Test scope: not deployed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>CI-0018</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>test/utils/mockOidc.js</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>RSA</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Deprecated/weak regardless of PQC</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>ML-DSA-87 (FIPS 204) or SLH-DSA (FIPS 205) for signatures</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
           <t>Keep for negative testing only; confirm the kid stays in the insecureKids denylist.</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>Phase 1</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="L22" s="2" t="inlineStr">
         <is>
           <t>Private key material is embedded in source; the key reproduces a known insecure IdP default key for negative tests. Test scope: not deployed.</t>
         </is>
@@ -17454,7 +18064,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-09-14T21:41:14+00:00</t>
+          <t>2026-09-14T21:51:24+00:00</t>
         </is>
       </c>
     </row>
@@ -17466,7 +18076,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>c066205075826a893833d9c1491589309c9bac32</t>
+          <t>a60a688755640584254099a89a37b16c2c221feb</t>
         </is>
       </c>
     </row>
@@ -17507,7 +18117,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7">
@@ -17559,7 +18169,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13">
@@ -17631,7 +18241,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21">
@@ -17753,7 +18363,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="34">
@@ -17825,7 +18435,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42">
@@ -17867,7 +18477,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="47">
@@ -18037,7 +18647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -18220,7 +18830,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Vendored third-party code (client/src/ext), minified bundles, lockfiles (except for version extraction), XCCDF/CKL STIG content fixtures (test/api/form-data-files, *.xml, *.ckl), generated docs, this scanner and its output directory are not pattern-scanned.</t>
+          <t>Vendored third-party code (client/src/ext), minified bundles, lockfiles (except for version extraction), XCCDF/CKL STIG content fixtures (test/api/form-data-files, *.xml, *.ckl), generated docs, this scanner and its output directory (the canonical docs/security/crypto-inventory and any in-repository --out path) are not pattern-scanned.</t>
         </is>
       </c>
     </row>
@@ -18232,7 +18842,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Prose in documentation is scanned only for configuration identifiers (environment variable names, TLS directives). Narrative mentions of algorithms in release notes or user guides are not inventoried.</t>
+          <t>Text PEM files with certificate/key extensions are parsed for metadata and also run through the pattern rules, so a committed private key appears both in the certificate table and as a Secret row. Binary keystores (.p12, .pfx, .jks) are recorded as not parsed.</t>
         </is>
       </c>
     </row>
@@ -18244,7 +18854,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Secret detection uses simple assignment patterns and JWT/JWK/PEM shapes. It will miss encoded or split secrets and may flag placeholder values used in tests; each Secret row is labeled with its scope (Test, CI, Documentation).</t>
+          <t>Prose in documentation is scanned only for configuration identifiers (environment variable names, TLS directives). Narrative mentions of algorithms in release notes or user guides are not inventoried.</t>
         </is>
       </c>
     </row>
@@ -18256,7 +18866,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>The `node:lts-alpine` tag and `lts/*` CI alias resolve to different Node versions over time. The resolved version is recorded only when supplied with --lts-resolves-to.</t>
+          <t>Secret detection uses simple assignment patterns and JWT/JWK/PEM shapes. It will miss encoded or split secrets and may flag placeholder values used in tests; each Secret row is labeled with its scope (Test, CI, Documentation).</t>
         </is>
       </c>
     </row>
@@ -18268,53 +18878,65 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Occurrences of the same JWT literal pattern inside a single test file are collapsed to one row (first line, count in the rationale).</t>
+          <t>The `node:lts-alpine` tag and `lts/*` CI alias resolve to different Node versions over time. The resolved version is recorded only when supplied with --lts-resolves-to.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Excluded</t>
+          <t>Limit</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Directories not scanned: .git, .nyc_output, .pytest_cache, __pycache__, _build, client/src/ext, coverage, dist, docs/security/crypto-inventory, mochawesome-report, node_modules, test/api/form-data-files, uploads</t>
+          <t>Occurrences of the same JWT literal pattern inside a single test file are collapsed to one row (first line, count in the rationale).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Parsers</t>
+          <t>Excluded</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>cryptography available: True; openssl CLI available: True</t>
+          <t>Directories not scanned: .git, .nyc_output, .pytest_cache, __pycache__, _build, client/src/ext, coverage, dist, docs/security/crypto-inventory, mochawesome-report, node_modules, test/api/form-data-files, uploads</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Classes</t>
+          <t>Parsers</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Quantum-vulnerability classes: Quantum-vulnerable (Shor) | Deprecated/weak regardless of PQC | Symmetric — Grover-affected, adequate at ≥256-bit | Protocol/configuration — inherits class of negotiated algorithms | Not applicable (no quantum-relevant primitive)</t>
+          <t>cryptography available: True; openssl CLI available: True</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>Classes</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Quantum-vulnerability classes: Quantum-vulnerable (Shor) | Deprecated/weak regardless of PQC | Symmetric — Grover-affected, adequate at ≥256-bit | Protocol/configuration — inherits class of negotiated algorithms | Not applicable (no quantum-relevant primitive)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>1 = act in Phase 1 (hygiene) or blocks later phases; 2 = Phase 1/2 configuration and TLS work; 3 = track, depends on external party or test-only; 4 = informational, no migration action.</t>
         </is>

</xml_diff>

<commit_message>
crypto-inventory: regenerate artifacts from 0ac904c6 (364 files, 57 rules, 144 rows)
Co-Authored-By: Erik Rozi <erik.rozi@cognition.ai>
</commit_message>
<xml_diff>
--- a/docs/security/crypto-inventory/Cryptographic-Inventory.xlsx
+++ b/docs/security/crypto-inventory/Cryptographic-Inventory.xlsx
@@ -18049,7 +18049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B62"/>
+  <dimension ref="A1:B63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -18064,7 +18064,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-09-14T21:51:24+00:00</t>
+          <t>2026-09-14T22:02:01+00:00</t>
         </is>
       </c>
     </row>
@@ -18076,290 +18076,292 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>a60a688755640584254099a89a37b16c2c221feb</t>
+          <t>0ac904c6c01e2ab14e783ecfa03588c8531870d2</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Files pattern-scanned</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>365</v>
+          <t>Source tree vs. commit</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>clean: scanned source equals HEAD</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Files skipped (binary/oversize/excluded type)</t>
+          <t>Files pattern-scanned</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>471</v>
+        <v>364</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Detection rules</t>
+          <t>Files skipped (binary/oversize/excluded type)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>51</v>
+        <v>469</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Inventory rows</t>
+          <t>Detection rules</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>144</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Certificates parsed</t>
+          <t>Inventory rows</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>144</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Certificate entries not parsed</t>
+          <t>Certificates parsed</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Certificate entries not parsed</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Libraries inventoried</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B10" t="n">
         <v>11</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Rows by quantum-vulnerability class</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Quantum-vulnerable (Shor)</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>17</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Deprecated/weak regardless of PQC</t>
+          <t>Quantum-vulnerable (Shor)</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Symmetric — Grover-affected, adequate at ≥256-bit</t>
+          <t>Deprecated/weak regardless of PQC</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Protocol/configuration — inherits class of negotiated algorithms</t>
+          <t>Symmetric — Grover-affected, adequate at ≥256-bit</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>Protocol/configuration — inherits class of negotiated algorithms</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Not applicable (no quantum-relevant primitive)</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B17" t="n">
         <v>81</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Rows by migration priority (1 = highest)</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>59</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B22" t="n">
+      <c r="B23" t="n">
         <v>69</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>Rows by category</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Asymmetric</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Certificate/Key material</t>
+          <t>Asymmetric</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Hash</t>
+          <t>Certificate/Key material</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>JWT/JWS/JWKS</t>
+          <t>Hash</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Randomness</t>
+          <t>JWT/JWS/JWKS</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Runtime</t>
+          <t>Randomness</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Secret</t>
+          <t>Runtime</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>53</v>
+        <v>9</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Secret reference</t>
+          <t>Secret</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>9</v>
+        <v>53</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Signing</t>
+          <t>Secret reference</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -18369,161 +18371,159 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>Signing</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>TLS</t>
         </is>
       </c>
-      <c r="B34" t="n">
+      <c r="B35" t="n">
         <v>32</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>Rows by scope</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>API (server)</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>32</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>API (server)</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Client (browser)</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>10</v>
+        <v>29</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Client (browser)</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Repository</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>Repository</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>Test</t>
         </is>
       </c>
-      <c r="B42" t="n">
+      <c r="B43" t="n">
         <v>51</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="3" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>Rows by crypto-agility rating</t>
         </is>
       </c>
-      <c r="B44" s="3" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Configurable</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>55</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Hardcoded</t>
+          <t>Configurable</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Library-bound</t>
+          <t>Hardcoded</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>5</v>
+        <v>75</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>Library-bound</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="B48" t="n">
+      <c r="B49" t="n">
         <v>9</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="3" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>Runtime pins found</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Dockerfile:15 (Node.js/OpenSSL runtime (container base image))</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>node:lts-alpine</t>
-        </is>
-      </c>
+      <c r="B51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>.github/workflows/api-container-tests.yml:40 (Node.js runtime (container test matrix))</t>
+          <t>Dockerfile:15 (Node.js/OpenSSL runtime (container base image))</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -18535,87 +18535,87 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>.github/workflows/api-container-tests.yml:40 (Node.js runtime (container test matrix))</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>node:lts-alpine</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>api/pkg.config.json:14 (Node.js runtime (packaged binaries))</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>node24-win,node24-linuxstatic</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="3" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>Local runtime probe (scanning host, not the deployed image)</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>node</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>24.19.0</t>
-        </is>
-      </c>
+      <c r="B56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>openssl</t>
+          <t>node</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>3.5.7</t>
+          <t>24.19.0</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>tls_default_min</t>
+          <t>openssl</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>TLSv1.2</t>
+          <t>3.5.7</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>tls_default_max</t>
+          <t>tls_default_min</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>TLSv1.3</t>
+          <t>TLSv1.2</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ml-kem-768</t>
+          <t>tls_default_max</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>available</t>
+          <t>TLSv1.3</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ml-dsa-65</t>
+          <t>ml-kem-768</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -18627,10 +18627,22 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
+          <t>ml-dsa-65</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
           <t>node:lts / lts/* resolution supplied at scan time</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>Node.js 24 (active LTS until 2026-10-28 per nodejs/Release schedule; bundles OpenSSL 3.5 from 24.5.0)</t>
         </is>
@@ -18647,7 +18659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -18686,7 +18698,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Context window of ±12 lines is inspected to infer key sizes (modulusLength, JWK `n` length), purpose (PKCE, kid derivation, attachment metadata), and presence/absence of TLS or JWT verification options.</t>
+          <t>Node.js crypto API calls are matched by name: generateKeyPair/Sync (rsa, rsa-pss, ec, ed25519, ed448, x25519, x448, dsa, dh), createECDH, diffieHellman, computeSecret, createDiffieHellman/Group, getDiffieHellman, createSign/createVerify, crypto.sign/verify, createCipheriv/createDecipheriv, and Web Crypto subtle.* calls with a public-key algorithm name. Curve, prime length and cipher name are taken from the literal arguments of the same call when present.</t>
         </is>
       </c>
     </row>
@@ -18698,7 +18710,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Certificate and key files by extension (.cer, .crt, .csr, .der, .jks, .key, .p12, .pem, .pfx) are parsed with `cryptography` or the `openssl` CLI.</t>
+          <t>Context window of ±12 lines is inspected to infer key sizes (modulusLength, JWK `n` length), purpose (PKCE, kid derivation, attachment metadata), and presence/absence of TLS or JWT verification options.</t>
         </is>
       </c>
     </row>
@@ -18710,7 +18722,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Embedded certificates and public keys are parsed from PEM blocks, JWKS `x5c` arrays and TUF/Notary root metadata (root.json).</t>
+          <t>Certificate and key files by extension (.cer, .crt, .csr, .der, .jks, .key, .p12, .pem, .pfx) are parsed with `cryptography` or the `openssl` CLI.</t>
         </is>
       </c>
     </row>
@@ -18722,7 +18734,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>package.json and package-lock.json files are read for declared and resolved versions of libraries with a cryptographic role.</t>
+          <t>Embedded certificates and public keys are parsed from PEM blocks, JWKS `x5c` arrays and TUF/Notary root metadata (root.json).</t>
         </is>
       </c>
     </row>
@@ -18734,7 +18746,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Dockerfiles, GitHub Actions workflows and pkg build configuration are read for Node.js runtime pins.</t>
+          <t>package.json and package-lock.json files are read for declared and resolved versions of libraries with a cryptographic role.</t>
         </is>
       </c>
     </row>
@@ -18746,7 +18758,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>If `node` is on PATH, the local runtime is probed for Node/OpenSSL versions, default TLS versions and ML-KEM/ML-DSA availability. This describes the scanning host, not the deployed container.</t>
+          <t>Dockerfiles, GitHub Actions workflows and pkg build configuration are read for Node.js runtime pins.</t>
         </is>
       </c>
     </row>
@@ -18758,7 +18770,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Secrets: only path, line and type are recorded; matched values are never written.</t>
+          <t>If `node` is on PATH, the local runtime is probed for Node/OpenSSL versions, default TLS versions and ML-KEM/ML-DSA availability. This describes the scanning host, not the deployed container.</t>
         </is>
       </c>
     </row>
@@ -18770,7 +18782,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Certificate subject/issuer: only attribute types and self-signed status are recorded unless --dn-values is given.</t>
+          <t>Secrets: only path, line and type are recorded; matched values are never written.</t>
         </is>
       </c>
     </row>
@@ -18782,19 +18794,19 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Absence checks: if no HSTS header and no explicit TLS option (minVersion, maxVersion, ciphers, rejectUnauthorized, secureOptions, honorCipherOrder, ecdhCurve) is found anywhere in scanned files, one row per absence is added and anchored to the TLS server setup line.</t>
+          <t>Certificate subject/issuer: only attribute types and self-signed status are recorded unless --dn-values is given.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Limit</t>
+          <t>Check</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Static text matching only. Dynamic algorithm selection (for example the algorithm list jsonwebtoken derives from the key type) is inferred from library source knowledge, not observed at runtime.</t>
+          <t>Absence checks: if no HSTS header and no explicit TLS option (minVersion, maxVersion, ciphers, rejectUnauthorized, secureOptions, honorCipherOrder, ecdhCurve) is found anywhere in scanned files, one row per absence is added and anchored to the TLS server setup line.</t>
         </is>
       </c>
     </row>
@@ -18806,7 +18818,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Key sizes are recorded only where they appear in source (modulusLength), can be derived from embedded key material (JWK `n`, SPKI), or are stated in comments. Keys supplied at deployment time (TLS certificates, IdP signing keys) are not visible to the scanner.</t>
+          <t>Static text matching only. Dynamic algorithm selection (for example the algorithm list jsonwebtoken derives from the key type) is inferred from library source knowledge, not observed at runtime.</t>
         </is>
       </c>
     </row>
@@ -18818,7 +18830,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>TLS protocol versions and cipher suites negotiated at runtime depend on the Node.js/OpenSSL build of the container image and on peers (reverse proxy, MySQL server, IdP, browsers). The scanner records what the repository configures and flags what it does not configure.</t>
+          <t>Key sizes are recorded only where they appear in source (modulusLength), can be derived from embedded key material (JWK `n`, SPKI), or are stated in comments. Keys supplied at deployment time (TLS certificates, IdP signing keys) are not visible to the scanner.</t>
         </is>
       </c>
     </row>
@@ -18830,7 +18842,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Vendored third-party code (client/src/ext), minified bundles, lockfiles (except for version extraction), XCCDF/CKL STIG content fixtures (test/api/form-data-files, *.xml, *.ckl), generated docs, this scanner and its output directory (the canonical docs/security/crypto-inventory and any in-repository --out path) are not pattern-scanned.</t>
+          <t>TLS protocol versions and cipher suites negotiated at runtime depend on the Node.js/OpenSSL build of the container image and on peers (reverse proxy, MySQL server, IdP, browsers). The scanner records what the repository configures and flags what it does not configure.</t>
         </is>
       </c>
     </row>
@@ -18842,7 +18854,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Text PEM files with certificate/key extensions are parsed for metadata and also run through the pattern rules, so a committed private key appears both in the certificate table and as a Secret row. Binary keystores (.p12, .pfx, .jks) are recorded as not parsed.</t>
+          <t>Vendored third-party code (client/src/ext), minified bundles, lockfiles (except for version extraction), XCCDF/CKL STIG content fixtures (test/api/form-data-files, *.xml, *.ckl), generated docs, this scanner and its output directory (the canonical docs/security/crypto-inventory and any in-repository --out path) are not pattern-scanned.</t>
         </is>
       </c>
     </row>
@@ -18854,7 +18866,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Prose in documentation is scanned only for configuration identifiers (environment variable names, TLS directives). Narrative mentions of algorithms in release notes or user guides are not inventoried.</t>
+          <t>Text PEM files with certificate/key extensions are parsed for metadata and also run through the pattern rules, so a committed private key appears both in the certificate table and as a Secret row. Binary keystores (.p12, .pfx, .jks) are recorded as not parsed.</t>
         </is>
       </c>
     </row>
@@ -18866,7 +18878,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Secret detection uses simple assignment patterns and JWT/JWK/PEM shapes. It will miss encoded or split secrets and may flag placeholder values used in tests; each Secret row is labeled with its scope (Test, CI, Documentation).</t>
+          <t>Prose in documentation is scanned only for configuration identifiers (environment variable names, TLS directives). Narrative mentions of algorithms in release notes or user guides are not inventoried.</t>
         </is>
       </c>
     </row>
@@ -18878,7 +18890,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>The `node:lts-alpine` tag and `lts/*` CI alias resolve to different Node versions over time. The resolved version is recorded only when supplied with --lts-resolves-to.</t>
+          <t>Secret detection uses simple assignment patterns and JWT/JWK/PEM shapes. It will miss encoded or split secrets and may flag placeholder values used in tests; each Secret row is labeled with its scope (Test, CI, Documentation).</t>
         </is>
       </c>
     </row>
@@ -18890,53 +18902,77 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Occurrences of the same JWT literal pattern inside a single test file are collapsed to one row (first line, count in the rationale).</t>
+          <t>The `node:lts-alpine` tag and `lts/*` CI alias resolve to different Node versions over time. The resolved version is recorded only when supplied with --lts-resolves-to.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Excluded</t>
+          <t>Limit</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Directories not scanned: .git, .nyc_output, .pytest_cache, __pycache__, _build, client/src/ext, coverage, dist, docs/security/crypto-inventory, mochawesome-report, node_modules, test/api/form-data-files, uploads</t>
+          <t>Occurrences of the same JWT literal pattern inside a single test file are collapsed to one row (first line, count in the rationale).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Parsers</t>
+          <t>Limit</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>cryptography available: True; openssl CLI available: True</t>
+          <t>`commit_sha` is HEAD of the checkout at scan time and `source_tree_vs_commit` records whether the scanned source matched it. Because the generated artifacts are committed on top of that source, the SHA recorded inside an artifact is always the parent of the commit that adds the artifact, never that commit itself.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Classes</t>
+          <t>Excluded</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Quantum-vulnerability classes: Quantum-vulnerable (Shor) | Deprecated/weak regardless of PQC | Symmetric — Grover-affected, adequate at ≥256-bit | Protocol/configuration — inherits class of negotiated algorithms | Not applicable (no quantum-relevant primitive)</t>
+          <t>Directories not scanned: .git, .mypy_cache, .nyc_output, .pytest_cache, .ruff_cache, .venv, __pycache__, _build, client/src/ext, coverage, dist, docs/security/crypto-inventory, mochawesome-report, node_modules, test/api/form-data-files, uploads, venv</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
+          <t>Parsers</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>cryptography available: True; openssl CLI available: True</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Classes</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Quantum-vulnerability classes: Quantum-vulnerable (Shor) | Deprecated/weak regardless of PQC | Symmetric — Grover-affected, adequate at ≥256-bit | Protocol/configuration — inherits class of negotiated algorithms | Not applicable (no quantum-relevant primitive)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>1 = act in Phase 1 (hygiene) or blocks later phases; 2 = Phase 1/2 configuration and TLS work; 3 = track, depends on external party or test-only; 4 = informational, no migration action.</t>
         </is>

</xml_diff>

<commit_message>
crypto-inventory: regenerate artifacts from 39981a0
Co-Authored-By: Erik Rozi <erik.rozi@cognition.ai>
</commit_message>
<xml_diff>
--- a/docs/security/crypto-inventory/Cryptographic-Inventory.xlsx
+++ b/docs/security/crypto-inventory/Cryptographic-Inventory.xlsx
@@ -18064,7 +18064,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-09-14T22:02:01+00:00</t>
+          <t>2026-09-14T22:10:31+00:00</t>
         </is>
       </c>
     </row>
@@ -18076,7 +18076,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0ac904c6c01e2ab14e783ecfa03588c8531870d2</t>
+          <t>39981a00c9e50c03b738062556a2eb050224704f</t>
         </is>
       </c>
     </row>
@@ -18722,7 +18722,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Certificate and key files by extension (.cer, .crt, .csr, .der, .jks, .key, .p12, .pem, .pfx) are parsed with `cryptography` or the `openssl` CLI.</t>
+          <t>Certificate and key files by extension (.cer, .crt, .csr, .der, .jks, .key, .p12, .pem, .pfx) are parsed with `cryptography` or the `openssl` CLI. PEM certificates give subject/issuer attribute types, key algorithm/size, signature algorithm and validity; PEM public keys and unencrypted private keys give key algorithm and size only (public parameters; private components are never read into the output). Encrypted keys, binary keystores and unreadable files are recorded as not parsed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
crypto-inventory: regenerate artifacts for 8cfef9d (58 rules, 144 rows unchanged)
Co-Authored-By: Erik Rozi <erik.rozi@cognition.ai>
</commit_message>
<xml_diff>
--- a/docs/security/crypto-inventory/Cryptographic-Inventory.xlsx
+++ b/docs/security/crypto-inventory/Cryptographic-Inventory.xlsx
@@ -18064,7 +18064,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-09-14T22:10:31+00:00</t>
+          <t>2026-09-14T22:21:52+00:00</t>
         </is>
       </c>
     </row>
@@ -18076,7 +18076,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>39981a00c9e50c03b738062556a2eb050224704f</t>
+          <t>8cfef9df0c6b1fea10450209e4639a74deb964e0</t>
         </is>
       </c>
     </row>
@@ -18119,7 +18119,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7">
@@ -18698,7 +18698,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Node.js crypto API calls are matched by name: generateKeyPair/Sync (rsa, rsa-pss, ec, ed25519, ed448, x25519, x448, dsa, dh), createECDH, diffieHellman, computeSecret, createDiffieHellman/Group, getDiffieHellman, createSign/createVerify, crypto.sign/verify, createCipheriv/createDecipheriv, and Web Crypto subtle.* calls with a public-key algorithm name. Curve, prime length and cipher name are taken from the literal arguments of the same call when present.</t>
+          <t>Node.js crypto API calls are matched by name: generateKeyPair/Sync (rsa, rsa-pss, ec, ed25519, ed448, x25519, x448, dsa, dh), createECDH, diffieHellman, computeSecret, createDiffieHellman/Group, getDiffieHellman, createSign/createVerify, crypto.sign/verify, createCipheriv/createDecipheriv, and Web Crypto subtle.* calls with a public-key algorithm name. Curve, prime length and cipher name are taken from the literal arguments of the same call when present. Call rules are matched against the call's first line plus the next 3 lines, so an argument list that continues on the following line is still inventoried once, at the line where the call starts.</t>
         </is>
       </c>
     </row>
@@ -18734,7 +18734,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Embedded certificates and public keys are parsed from PEM blocks, JWKS `x5c` arrays and TUF/Notary root metadata (root.json).</t>
+          <t>PEM blocks (certificate, public key, private key) found in any scanned text file are parsed the same way and the parsed algorithm, size, signature algorithm and validity are copied into the KEYMAT-PEM-* inventory row; RSA/DSA below 2048 bits and SHA-1/MD5 certificate signatures are classified as deprecated/weak. Blocks that cannot be parsed keep the block-type classification and say so in the Mode column. Public keys are also parsed from JWKS `x5c` arrays and TUF/Notary root metadata (root.json).</t>
         </is>
       </c>
     </row>
@@ -18854,7 +18854,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Vendored third-party code (client/src/ext), minified bundles, lockfiles (except for version extraction), XCCDF/CKL STIG content fixtures (test/api/form-data-files, *.xml, *.ckl), generated docs, this scanner and its output directory (the canonical docs/security/crypto-inventory and any in-repository --out path) are not pattern-scanned.</t>
+          <t>Vendored third-party code (client/src/ext), minified bundles, lockfiles (except for version extraction), XCCDF/CKL STIG content fixtures (test/api/form-data-files, *.xml, *.ckl), generated docs, this scanner and its own output (the canonical docs/security/crypto-inventory directory, any in-repository --out directory, and the concrete JSON/XLSX/report/template output paths, so that `--out .` does not inventory the previous run) are not pattern-scanned.</t>
         </is>
       </c>
     </row>
@@ -18866,7 +18866,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Text PEM files with certificate/key extensions are parsed for metadata and also run through the pattern rules, so a committed private key appears both in the certificate table and as a Secret row. Binary keystores (.p12, .pfx, .jks) are recorded as not parsed.</t>
+          <t>Text PEM files with certificate/key extensions are parsed for metadata and also run through the pattern rules, so a committed private key appears both in the certificate table and as a Secret row. A PEM block may span at most 400 lines; longer blocks are recorded as not parsed. Binary keystores (.p12, .pfx, .jks) are recorded as not parsed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
crypto-inventory: regenerate artifacts for 4da8062 (62 rules, 144 rows unchanged)
Co-Authored-By: Erik Rozi <erik.rozi@cognition.ai>
</commit_message>
<xml_diff>
--- a/docs/security/crypto-inventory/Cryptographic-Inventory.xlsx
+++ b/docs/security/crypto-inventory/Cryptographic-Inventory.xlsx
@@ -18064,7 +18064,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-09-14T22:21:52+00:00</t>
+          <t>2026-09-14T22:31:45+00:00</t>
         </is>
       </c>
     </row>
@@ -18076,7 +18076,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>8cfef9df0c6b1fea10450209e4639a74deb964e0</t>
+          <t>4da806210cd254dbf8c9e20b8d85bcbe564a2323</t>
         </is>
       </c>
     </row>
@@ -18119,7 +18119,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7">
@@ -18135,7 +18135,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Certificates parsed</t>
+          <t>Certificate/key entries parsed</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -18145,7 +18145,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Certificate entries not parsed</t>
+          <t>Certificate/key entries not parsed</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -18722,7 +18722,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Certificate and key files by extension (.cer, .crt, .csr, .der, .jks, .key, .p12, .pem, .pfx) are parsed with `cryptography` or the `openssl` CLI. PEM certificates give subject/issuer attribute types, key algorithm/size, signature algorithm and validity; PEM public keys and unencrypted private keys give key algorithm and size only (public parameters; private components are never read into the output). Encrypted keys, binary keystores and unreadable files are recorded as not parsed.</t>
+          <t>Certificate and key files by extension (.cer, .crt, .csr, .der, .jks, .key, .p12, .pem, .pfx) are parsed with `cryptography` or the `openssl` CLI. PEM certificates give subject/issuer attribute types, key algorithm/size, signature algorithm and validity; PEM public keys and unencrypted private keys give key algorithm and size only (public parameters; private components are never read into the output). Files without a PEM block are tried as DER certificate, then DER private key, then DER public key, and get a KEYMAT-DER-* inventory row; keystores and files that parse as none of these get a KEYMAT-FILE-UNPARSED row (priority 2) and are recorded as not parsed. Encrypted keys and unreadable files are recorded as not parsed.</t>
         </is>
       </c>
     </row>
@@ -18866,7 +18866,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Text PEM files with certificate/key extensions are parsed for metadata and also run through the pattern rules, so a committed private key appears both in the certificate table and as a Secret row. A PEM block may span at most 400 lines; longer blocks are recorded as not parsed. Binary keystores (.p12, .pfx, .jks) are recorded as not parsed.</t>
+          <t>Text PEM files with certificate/key extensions are parsed for metadata and also run through the pattern rules, so a committed private key appears both in the certificate table and as a Secret row. A PEM block may span at most 400 lines; longer blocks are recorded as not parsed. Binary keystores (.p12, .pfx, .jks) are inventoried by path only; their contents are not parsed (password required).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
crypto-inventory: regenerate artifacts for 781f8a6 (64 rules, 144 rows unchanged)
Co-Authored-By: Erik Rozi <erik.rozi@cognition.ai>
</commit_message>
<xml_diff>
--- a/docs/security/crypto-inventory/Cryptographic-Inventory.xlsx
+++ b/docs/security/crypto-inventory/Cryptographic-Inventory.xlsx
@@ -3065,12 +3065,12 @@
       <c r="G27" s="2" t="inlineStr"/>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>No Strict-Transport-Security header or helmet() use in application code; browsers are not instructed to require HTTPS by the API itself.</t>
+          <t>No Strict-Transport-Security header or helmet() use in application code or deployable configuration (documentation, tests and CI excluded); browsers are not instructed to require HTTPS by the API itself.</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Absence check across all scanned files</t>
+          <t>Absence check across application code and deployable configuration</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="U27" s="2" t="inlineStr">
         <is>
-          <t>pattern not found in any scanned file</t>
+          <t>pattern not found in any API, client or repository-level file</t>
         </is>
       </c>
       <c r="V27" s="2" t="inlineStr">
@@ -3169,12 +3169,12 @@
       <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>No minVersion, maxVersion, ciphers, rejectUnauthorized, secureOptions, honorCipherOrder or ecdhCurve literal anywhere in scanned files. Node.js defaults apply to the API server, the MySQL client and the IdP clients.</t>
+          <t>No minVersion, maxVersion, ciphers, rejectUnauthorized, secureOptions, honorCipherOrder or ecdhCurve literal in application code or deployable configuration (documentation, tests and CI excluded). Node.js defaults apply to the API server, the MySQL client and the IdP clients.</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Absence check across all scanned files</t>
+          <t>Absence check across application code and deployable configuration</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="U28" s="2" t="inlineStr">
         <is>
-          <t>pattern not found in any scanned file</t>
+          <t>pattern not found in any API, client or repository-level file</t>
         </is>
       </c>
       <c r="V28" s="2" t="inlineStr">
@@ -14058,12 +14058,12 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>No Strict-Transport-Security header or helmet() use in application code; browsers are not instructed to require HTTPS by the API itself.</t>
+          <t>No Strict-Transport-Security header or helmet() use in application code or deployable configuration (documentation, tests and CI excluded); browsers are not instructed to require HTTPS by the API itself.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Absence check across all scanned files</t>
+          <t>Absence check across application code and deployable configuration</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -14106,12 +14106,12 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>No minVersion, maxVersion, ciphers, rejectUnauthorized, secureOptions, honorCipherOrder or ecdhCurve literal anywhere in scanned files. Node.js defaults apply to the API server, the MySQL client and the IdP clients.</t>
+          <t>No minVersion, maxVersion, ciphers, rejectUnauthorized, secureOptions, honorCipherOrder or ecdhCurve literal in application code or deployable configuration (documentation, tests and CI excluded). Node.js defaults apply to the API server, the MySQL client and the IdP clients.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Absence check across all scanned files</t>
+          <t>Absence check across application code and deployable configuration</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -16454,7 +16454,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>No Strict-Transport-Security header or helmet() use in application code; browsers are not instructed to require HTTPS by the API itself.</t>
+          <t>No Strict-Transport-Security header or helmet() use in application code or deployable configuration (documentation, tests and CI excluded); browsers are not instructed to require HTTPS by the API itself.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -16494,7 +16494,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>No minVersion, maxVersion, ciphers, rejectUnauthorized, secureOptions, honorCipherOrder or ecdhCurve literal anywhere in scanned files. Node.js defaults apply to the API server, the MySQL client and the IdP clients.</t>
+          <t>No minVersion, maxVersion, ciphers, rejectUnauthorized, secureOptions, honorCipherOrder or ecdhCurve literal in application code or deployable configuration (documentation, tests and CI excluded). Node.js defaults apply to the API server, the MySQL client and the IdP clients.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -18064,7 +18064,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-09-14T22:31:45+00:00</t>
+          <t>2026-09-14T22:46:02+00:00</t>
         </is>
       </c>
     </row>
@@ -18076,7 +18076,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>4da806210cd254dbf8c9e20b8d85bcbe564a2323</t>
+          <t>781f8a6e5ee67c9822f98f46f3cb9c3e155d7d13</t>
         </is>
       </c>
     </row>
@@ -18119,7 +18119,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7">
@@ -18659,7 +18659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -18710,7 +18710,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Context window of ±12 lines is inspected to infer key sizes (modulusLength, JWK `n` length), purpose (PKCE, kid derivation, attachment metadata), and presence/absence of TLS or JWT verification options.</t>
+          <t>Password hashing and KDF calls are matched as package calls or methods (bcrypt/bcryptjs/argon2 followed by any method such as hash, hashSync, compare, verify, including optional chaining), as node:crypto functions (pbkdf2/Sync, scrypt/Sync, hkdf/Sync) and as Web Crypto deriveBits/deriveKey/importKey with PBKDF2 or HKDF. Aliased imports (`const h = bcrypt.hash`, `import { hash } from 'bcrypt'`) are not followed.</t>
         </is>
       </c>
     </row>
@@ -18722,7 +18722,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Certificate and key files by extension (.cer, .crt, .csr, .der, .jks, .key, .p12, .pem, .pfx) are parsed with `cryptography` or the `openssl` CLI. PEM certificates give subject/issuer attribute types, key algorithm/size, signature algorithm and validity; PEM public keys and unencrypted private keys give key algorithm and size only (public parameters; private components are never read into the output). Files without a PEM block are tried as DER certificate, then DER private key, then DER public key, and get a KEYMAT-DER-* inventory row; keystores and files that parse as none of these get a KEYMAT-FILE-UNPARSED row (priority 2) and are recorded as not parsed. Encrypted keys and unreadable files are recorded as not parsed.</t>
+          <t>Secret literals are matched as quoted assignments in any text file and as unquoted scalars only in dotenv, shell, YAML, properties, ini, conf, toml and Dockerfile inputs, where an unquoted value is a literal rather than an identifier; values starting with $, %, {, *, &amp;, &lt; or ( are treated as references or placeholders.</t>
         </is>
       </c>
     </row>
@@ -18734,7 +18734,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>PEM blocks (certificate, public key, private key) found in any scanned text file are parsed the same way and the parsed algorithm, size, signature algorithm and validity are copied into the KEYMAT-PEM-* inventory row; RSA/DSA below 2048 bits and SHA-1/MD5 certificate signatures are classified as deprecated/weak. Blocks that cannot be parsed keep the block-type classification and say so in the Mode column. Public keys are also parsed from JWKS `x5c` arrays and TUF/Notary root metadata (root.json).</t>
+          <t>Context window of ±12 lines is inspected to infer key sizes (modulusLength, JWK `n` length), purpose (PKCE, kid derivation, attachment metadata), and presence/absence of TLS or JWT verification options.</t>
         </is>
       </c>
     </row>
@@ -18746,7 +18746,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>package.json and package-lock.json files are read for declared and resolved versions of libraries with a cryptographic role.</t>
+          <t>Certificate and key files by extension (.cer, .crt, .csr, .der, .jks, .key, .p12, .pem, .pfx) are parsed with `cryptography` or the `openssl` CLI. PEM certificates give subject/issuer attribute types, key algorithm/size, signature algorithm and validity; PEM public keys and unencrypted private keys give key algorithm and size only (public parameters; private components are never read into the output). Files without a PEM block are tried as DER certificate, then DER private key, then DER public key, and get a KEYMAT-DER-* inventory row; keystores and files that parse as none of these get a KEYMAT-FILE-UNPARSED row (priority 2) and are recorded as not parsed. Encrypted keys and unreadable files are recorded as not parsed.</t>
         </is>
       </c>
     </row>
@@ -18758,7 +18758,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Dockerfiles, GitHub Actions workflows and pkg build configuration are read for Node.js runtime pins.</t>
+          <t>PEM blocks (certificate, public key, private key) found in any scanned text file are parsed the same way and the parsed algorithm, size, signature algorithm and validity are copied into the KEYMAT-PEM-* inventory row; RSA/DSA below 2048 bits and SHA-1/MD5 certificate signatures are classified as deprecated/weak. Blocks that cannot be parsed keep the block-type classification and say so in the Mode column. Public keys are also parsed from JWKS `x5c` arrays and TUF/Notary root metadata (root.json).</t>
         </is>
       </c>
     </row>
@@ -18770,7 +18770,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>If `node` is on PATH, the local runtime is probed for Node/OpenSSL versions, default TLS versions and ML-KEM/ML-DSA availability. This describes the scanning host, not the deployed container.</t>
+          <t>package.json and package-lock.json files are read for declared and resolved versions of libraries with a cryptographic role.</t>
         </is>
       </c>
     </row>
@@ -18782,7 +18782,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Secrets: only path, line and type are recorded; matched values are never written.</t>
+          <t>Dockerfiles, GitHub Actions workflows and pkg build configuration are read for Node.js runtime pins.</t>
         </is>
       </c>
     </row>
@@ -18794,7 +18794,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Certificate subject/issuer: only attribute types and self-signed status are recorded unless --dn-values is given.</t>
+          <t>If `node` is on PATH, the local runtime is probed for Node/OpenSSL versions, default TLS versions and ML-KEM/ML-DSA availability. This describes the scanning host, not the deployed container.</t>
         </is>
       </c>
     </row>
@@ -18806,31 +18806,31 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Absence checks: if no HSTS header and no explicit TLS option (minVersion, maxVersion, ciphers, rejectUnauthorized, secureOptions, honorCipherOrder, ecdhCurve) is found anywhere in scanned files, one row per absence is added and anchored to the TLS server setup line.</t>
+          <t>Secrets: only path, line and type are recorded; matched values are never written.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Limit</t>
+          <t>Check</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Static text matching only. Dynamic algorithm selection (for example the algorithm list jsonwebtoken derives from the key type) is inferred from library source knowledge, not observed at runtime.</t>
+          <t>Certificate subject/issuer: only attribute types and self-signed status are recorded unless --dn-values is given.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Limit</t>
+          <t>Check</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Key sizes are recorded only where they appear in source (modulusLength), can be derived from embedded key material (JWK `n`, SPKI), or are stated in comments. Keys supplied at deployment time (TLS certificates, IdP signing keys) are not visible to the scanner.</t>
+          <t>Absence checks: if no HSTS header and no explicit TLS option (minVersion, maxVersion, ciphers, rejectUnauthorized, secureOptions, honorCipherOrder, ecdhCurve) is found in a file of scope API (server), Client (browser) or Repository, one row per absence is added and anchored to the TLS server setup line. Matches in Documentation, Test and CI scope are inventoried but do not satisfy the check, because prose describing a control does not configure it.</t>
         </is>
       </c>
     </row>
@@ -18842,7 +18842,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>TLS protocol versions and cipher suites negotiated at runtime depend on the Node.js/OpenSSL build of the container image and on peers (reverse proxy, MySQL server, IdP, browsers). The scanner records what the repository configures and flags what it does not configure.</t>
+          <t>Static text matching only. Dynamic algorithm selection (for example the algorithm list jsonwebtoken derives from the key type) is inferred from library source knowledge, not observed at runtime.</t>
         </is>
       </c>
     </row>
@@ -18854,7 +18854,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Vendored third-party code (client/src/ext), minified bundles, lockfiles (except for version extraction), XCCDF/CKL STIG content fixtures (test/api/form-data-files, *.xml, *.ckl), generated docs, this scanner and its own output (the canonical docs/security/crypto-inventory directory, any in-repository --out directory, and the concrete JSON/XLSX/report/template output paths, so that `--out .` does not inventory the previous run) are not pattern-scanned.</t>
+          <t>Key sizes are recorded only where they appear in source (modulusLength), can be derived from embedded key material (JWK `n`, SPKI), or are stated in comments. Keys supplied at deployment time (TLS certificates, IdP signing keys) are not visible to the scanner.</t>
         </is>
       </c>
     </row>
@@ -18866,7 +18866,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Text PEM files with certificate/key extensions are parsed for metadata and also run through the pattern rules, so a committed private key appears both in the certificate table and as a Secret row. A PEM block may span at most 400 lines; longer blocks are recorded as not parsed. Binary keystores (.p12, .pfx, .jks) are inventoried by path only; their contents are not parsed (password required).</t>
+          <t>TLS protocol versions and cipher suites negotiated at runtime depend on the Node.js/OpenSSL build of the container image and on peers (reverse proxy, MySQL server, IdP, browsers). The scanner records what the repository configures and flags what it does not configure.</t>
         </is>
       </c>
     </row>
@@ -18878,7 +18878,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Prose in documentation is scanned only for configuration identifiers (environment variable names, TLS directives). Narrative mentions of algorithms in release notes or user guides are not inventoried.</t>
+          <t>Vendored third-party code (client/src/ext), minified bundles, lockfiles (except for version extraction), XCCDF/CKL STIG content fixtures (test/api/form-data-files, *.xml, *.ckl), generated docs, this scanner and its own output (the canonical docs/security/crypto-inventory directory, any in-repository --out directory, and the concrete JSON/XLSX/report/template output paths, so that `--out .` does not inventory the previous run) are not pattern-scanned.</t>
         </is>
       </c>
     </row>
@@ -18890,7 +18890,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Secret detection uses simple assignment patterns and JWT/JWK/PEM shapes. It will miss encoded or split secrets and may flag placeholder values used in tests; each Secret row is labeled with its scope (Test, CI, Documentation).</t>
+          <t>Text PEM files with certificate/key extensions are parsed for metadata and also run through the pattern rules, so a committed private key appears both in the certificate table and as a Secret row. A PEM block may span at most 400 lines; longer blocks are recorded as not parsed. Binary keystores (.p12, .pfx, .jks) are inventoried by path only; their contents are not parsed (password required).</t>
         </is>
       </c>
     </row>
@@ -18902,7 +18902,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>The `node:lts-alpine` tag and `lts/*` CI alias resolve to different Node versions over time. The resolved version is recorded only when supplied with --lts-resolves-to.</t>
+          <t>Prose in documentation is scanned only for configuration identifiers (environment variable names, TLS directives). Narrative mentions of algorithms in release notes or user guides are not inventoried.</t>
         </is>
       </c>
     </row>
@@ -18914,7 +18914,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Occurrences of the same JWT literal pattern inside a single test file are collapsed to one row (first line, count in the rationale).</t>
+          <t>Secret detection uses simple assignment patterns and JWT/JWK/PEM shapes. It will miss encoded or split secrets and may flag placeholder values used in tests; each Secret row is labeled with its scope (Test, CI, Documentation).</t>
         </is>
       </c>
     </row>
@@ -18926,53 +18926,77 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>`commit_sha` is HEAD of the checkout at scan time and `source_tree_vs_commit` records whether the scanned source matched it. Because the generated artifacts are committed on top of that source, the SHA recorded inside an artifact is always the parent of the commit that adds the artifact, never that commit itself.</t>
+          <t>The `node:lts-alpine` tag and `lts/*` CI alias resolve to different Node versions over time. The resolved version is recorded only when supplied with --lts-resolves-to.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Excluded</t>
+          <t>Limit</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Directories not scanned: .git, .mypy_cache, .nyc_output, .pytest_cache, .ruff_cache, .venv, __pycache__, _build, client/src/ext, coverage, dist, docs/security/crypto-inventory, mochawesome-report, node_modules, test/api/form-data-files, uploads, venv</t>
+          <t>Occurrences of the same JWT literal pattern inside a single test file are collapsed to one row (first line, count in the rationale).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Parsers</t>
+          <t>Limit</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>cryptography available: True; openssl CLI available: True</t>
+          <t>`commit_sha` is HEAD of the checkout at scan time and `source_tree_vs_commit` records whether the scanned source matched it. Because the generated artifacts are committed on top of that source, the SHA recorded inside an artifact is always the parent of the commit that adds the artifact, never that commit itself.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Classes</t>
+          <t>Excluded</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Quantum-vulnerability classes: Quantum-vulnerable (Shor) | Deprecated/weak regardless of PQC | Symmetric — Grover-affected, adequate at ≥256-bit | Protocol/configuration — inherits class of negotiated algorithms | Not applicable (no quantum-relevant primitive)</t>
+          <t>Directories not scanned: .git, .mypy_cache, .nyc_output, .pytest_cache, .ruff_cache, .venv, __pycache__, _build, client/src/ext, coverage, dist, docs/security/crypto-inventory, mochawesome-report, node_modules, test/api/form-data-files, uploads, venv</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t>Parsers</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>cryptography available: True; openssl CLI available: True</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Classes</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Quantum-vulnerability classes: Quantum-vulnerable (Shor) | Deprecated/weak regardless of PQC | Symmetric — Grover-affected, adequate at ≥256-bit | Protocol/configuration — inherits class of negotiated algorithms | Not applicable (no quantum-relevant primitive)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>1 = act in Phase 1 (hygiene) or blocks later phases; 2 = Phase 1/2 configuration and TLS work; 3 = track, depends on external party or test-only; 4 = informational, no migration action.</t>
         </is>

</xml_diff>

<commit_message>
crypto-inventory: regenerate artifacts at e426316
Method limits now document value-based weak classification and the
secureProtocol option; counts unchanged (144 rows, 364 files, 64 rules).

Co-Authored-By: Erik Rozi <erik.rozi@cognition.ai>
</commit_message>
<xml_diff>
--- a/docs/security/crypto-inventory/Cryptographic-Inventory.xlsx
+++ b/docs/security/crypto-inventory/Cryptographic-Inventory.xlsx
@@ -18064,7 +18064,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-09-14T22:46:02+00:00</t>
+          <t>2026-09-14T22:57:35+00:00</t>
         </is>
       </c>
     </row>
@@ -18076,7 +18076,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>781f8a6e5ee67c9822f98f46f3cb9c3e155d7d13</t>
+          <t>e426316e995d04bff8ea7cdeb6803e5abce6dec1</t>
         </is>
       </c>
     </row>
@@ -18659,7 +18659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -18734,7 +18734,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Context window of ±12 lines is inspected to infer key sizes (modulusLength, JWK `n` length), purpose (PKCE, kid derivation, attachment metadata), and presence/absence of TLS or JWT verification options.</t>
+          <t>Literal values decide the weak class, not only the option or API name: minVersion/maxVersion/secureProtocol below TLS 1.2 (SSLv2, SSLv3, TLSv1, TLSv1.1 and the *_method constants), cipher lists that enable RC4, DES/3DES, NULL, export or MD5 suites, createSign/createVerify/crypto.sign/verify and Web Crypto `hash:` parameters naming MD5 or SHA-1, createHmac('md5'), and createCipheriv names for DES, RC2, RC4, Blowfish, IDEA, SEED or CAST are classified `Deprecated/weak regardless of PQC` at priority 1. `rejectUnauthorized: false` keeps the protocol class but is raised to priority 1 with a stated gap. HMAC-SHA-1 stays in the Grover class (acceptable under SP 800-131A Rev. 2). JWK fields are matched in both JavaScript (`d: '...'`) and JSON (`"d": "..."`) spelling.</t>
         </is>
       </c>
     </row>
@@ -18746,7 +18746,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Certificate and key files by extension (.cer, .crt, .csr, .der, .jks, .key, .p12, .pem, .pfx) are parsed with `cryptography` or the `openssl` CLI. PEM certificates give subject/issuer attribute types, key algorithm/size, signature algorithm and validity; PEM public keys and unencrypted private keys give key algorithm and size only (public parameters; private components are never read into the output). Files without a PEM block are tried as DER certificate, then DER private key, then DER public key, and get a KEYMAT-DER-* inventory row; keystores and files that parse as none of these get a KEYMAT-FILE-UNPARSED row (priority 2) and are recorded as not parsed. Encrypted keys and unreadable files are recorded as not parsed.</t>
+          <t>Context window of ±12 lines is inspected to infer key sizes (modulusLength, JWK `n` length), purpose (PKCE, kid derivation, attachment metadata), and presence/absence of TLS or JWT verification options.</t>
         </is>
       </c>
     </row>
@@ -18758,7 +18758,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>PEM blocks (certificate, public key, private key) found in any scanned text file are parsed the same way and the parsed algorithm, size, signature algorithm and validity are copied into the KEYMAT-PEM-* inventory row; RSA/DSA below 2048 bits and SHA-1/MD5 certificate signatures are classified as deprecated/weak. Blocks that cannot be parsed keep the block-type classification and say so in the Mode column. Public keys are also parsed from JWKS `x5c` arrays and TUF/Notary root metadata (root.json).</t>
+          <t>Certificate and key files by extension (.cer, .crt, .csr, .der, .jks, .key, .p12, .pem, .pfx) are parsed with `cryptography` or the `openssl` CLI. PEM certificates give subject/issuer attribute types, key algorithm/size, signature algorithm and validity; PEM public keys and unencrypted private keys give key algorithm and size only (public parameters; private components are never read into the output). Files without a PEM block are tried as DER certificate, then DER private key, then DER public key, and get a KEYMAT-DER-* inventory row; keystores and files that parse as none of these get a KEYMAT-FILE-UNPARSED row (priority 2) and are recorded as not parsed. Encrypted keys and unreadable files are recorded as not parsed.</t>
         </is>
       </c>
     </row>
@@ -18770,7 +18770,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>package.json and package-lock.json files are read for declared and resolved versions of libraries with a cryptographic role.</t>
+          <t>PEM blocks (certificate, public key, private key) found in any scanned text file are parsed the same way and the parsed algorithm, size, signature algorithm and validity are copied into the KEYMAT-PEM-* inventory row; RSA/DSA below 2048 bits and SHA-1/MD5 certificate signatures are classified as deprecated/weak. Blocks that cannot be parsed keep the block-type classification and say so in the Mode column. Public keys are also parsed from JWKS `x5c` arrays and TUF/Notary root metadata (root.json).</t>
         </is>
       </c>
     </row>
@@ -18782,7 +18782,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Dockerfiles, GitHub Actions workflows and pkg build configuration are read for Node.js runtime pins.</t>
+          <t>package.json and package-lock.json files are read for declared and resolved versions of libraries with a cryptographic role.</t>
         </is>
       </c>
     </row>
@@ -18794,7 +18794,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>If `node` is on PATH, the local runtime is probed for Node/OpenSSL versions, default TLS versions and ML-KEM/ML-DSA availability. This describes the scanning host, not the deployed container.</t>
+          <t>Dockerfiles, GitHub Actions workflows and pkg build configuration are read for Node.js runtime pins.</t>
         </is>
       </c>
     </row>
@@ -18806,7 +18806,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Secrets: only path, line and type are recorded; matched values are never written.</t>
+          <t>If `node` is on PATH, the local runtime is probed for Node/OpenSSL versions, default TLS versions and ML-KEM/ML-DSA availability. This describes the scanning host, not the deployed container.</t>
         </is>
       </c>
     </row>
@@ -18818,7 +18818,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Certificate subject/issuer: only attribute types and self-signed status are recorded unless --dn-values is given.</t>
+          <t>Secrets: only path, line and type are recorded; matched values are never written.</t>
         </is>
       </c>
     </row>
@@ -18830,19 +18830,19 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Absence checks: if no HSTS header and no explicit TLS option (minVersion, maxVersion, ciphers, rejectUnauthorized, secureOptions, honorCipherOrder, ecdhCurve) is found in a file of scope API (server), Client (browser) or Repository, one row per absence is added and anchored to the TLS server setup line. Matches in Documentation, Test and CI scope are inventoried but do not satisfy the check, because prose describing a control does not configure it.</t>
+          <t>Certificate subject/issuer: only attribute types and self-signed status are recorded unless --dn-values is given.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Limit</t>
+          <t>Check</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Static text matching only. Dynamic algorithm selection (for example the algorithm list jsonwebtoken derives from the key type) is inferred from library source knowledge, not observed at runtime.</t>
+          <t>Absence checks: if no HSTS header and no explicit TLS option (minVersion, maxVersion, secureProtocol, ciphers, rejectUnauthorized, secureOptions, honorCipherOrder, ecdhCurve) is found in a file of scope API (server), Client (browser) or Repository, one row per absence is added and anchored to the TLS server setup line. Matches in Documentation, Test and CI scope are inventoried but do not satisfy the check, because prose describing a control does not configure it.</t>
         </is>
       </c>
     </row>
@@ -18854,7 +18854,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Key sizes are recorded only where they appear in source (modulusLength), can be derived from embedded key material (JWK `n`, SPKI), or are stated in comments. Keys supplied at deployment time (TLS certificates, IdP signing keys) are not visible to the scanner.</t>
+          <t>Static text matching only. Dynamic algorithm selection (for example the algorithm list jsonwebtoken derives from the key type) is inferred from library source knowledge, not observed at runtime.</t>
         </is>
       </c>
     </row>
@@ -18866,7 +18866,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>TLS protocol versions and cipher suites negotiated at runtime depend on the Node.js/OpenSSL build of the container image and on peers (reverse proxy, MySQL server, IdP, browsers). The scanner records what the repository configures and flags what it does not configure.</t>
+          <t>Key sizes are recorded only where they appear in source (modulusLength), can be derived from embedded key material (JWK `n`, SPKI), or are stated in comments. Keys supplied at deployment time (TLS certificates, IdP signing keys) are not visible to the scanner.</t>
         </is>
       </c>
     </row>
@@ -18878,7 +18878,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Vendored third-party code (client/src/ext), minified bundles, lockfiles (except for version extraction), XCCDF/CKL STIG content fixtures (test/api/form-data-files, *.xml, *.ckl), generated docs, this scanner and its own output (the canonical docs/security/crypto-inventory directory, any in-repository --out directory, and the concrete JSON/XLSX/report/template output paths, so that `--out .` does not inventory the previous run) are not pattern-scanned.</t>
+          <t>TLS protocol versions and cipher suites negotiated at runtime depend on the Node.js/OpenSSL build of the container image and on peers (reverse proxy, MySQL server, IdP, browsers). The scanner records what the repository configures and flags what it does not configure.</t>
         </is>
       </c>
     </row>
@@ -18890,7 +18890,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Text PEM files with certificate/key extensions are parsed for metadata and also run through the pattern rules, so a committed private key appears both in the certificate table and as a Secret row. A PEM block may span at most 400 lines; longer blocks are recorded as not parsed. Binary keystores (.p12, .pfx, .jks) are inventoried by path only; their contents are not parsed (password required).</t>
+          <t>Vendored third-party code (client/src/ext), minified bundles, lockfiles (except for version extraction), XCCDF/CKL STIG content fixtures (test/api/form-data-files, *.xml, *.ckl), generated docs, this scanner and its own output (the canonical docs/security/crypto-inventory directory, any in-repository --out directory, and the concrete JSON/XLSX/report/template output paths, so that `--out .` does not inventory the previous run) are not pattern-scanned.</t>
         </is>
       </c>
     </row>
@@ -18902,7 +18902,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Prose in documentation is scanned only for configuration identifiers (environment variable names, TLS directives). Narrative mentions of algorithms in release notes or user guides are not inventoried.</t>
+          <t>Text PEM files with certificate/key extensions are parsed for metadata and also run through the pattern rules, so a committed private key appears both in the certificate table and as a Secret row. A PEM block may span at most 400 lines; longer blocks are recorded as not parsed. Binary keystores (.p12, .pfx, .jks) are inventoried by path only; their contents are not parsed (password required).</t>
         </is>
       </c>
     </row>
@@ -18914,7 +18914,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Secret detection uses simple assignment patterns and JWT/JWK/PEM shapes. It will miss encoded or split secrets and may flag placeholder values used in tests; each Secret row is labeled with its scope (Test, CI, Documentation).</t>
+          <t>Prose in documentation is scanned only for configuration identifiers (environment variable names, TLS directives). Narrative mentions of algorithms in release notes or user guides are not inventoried.</t>
         </is>
       </c>
     </row>
@@ -18926,7 +18926,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>The `node:lts-alpine` tag and `lts/*` CI alias resolve to different Node versions over time. The resolved version is recorded only when supplied with --lts-resolves-to.</t>
+          <t>Secret detection uses simple assignment patterns and JWT/JWK/PEM shapes. It will miss encoded or split secrets and may flag placeholder values used in tests; each Secret row is labeled with its scope (Test, CI, Documentation).</t>
         </is>
       </c>
     </row>
@@ -18938,7 +18938,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Occurrences of the same JWT literal pattern inside a single test file are collapsed to one row (first line, count in the rationale).</t>
+          <t>The `node:lts-alpine` tag and `lts/*` CI alias resolve to different Node versions over time. The resolved version is recorded only when supplied with --lts-resolves-to.</t>
         </is>
       </c>
     </row>
@@ -18950,53 +18950,65 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>`commit_sha` is HEAD of the checkout at scan time and `source_tree_vs_commit` records whether the scanned source matched it. Because the generated artifacts are committed on top of that source, the SHA recorded inside an artifact is always the parent of the commit that adds the artifact, never that commit itself.</t>
+          <t>Occurrences of the same JWT literal pattern inside a single test file are collapsed to one row (first line, count in the rationale).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Excluded</t>
+          <t>Limit</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Directories not scanned: .git, .mypy_cache, .nyc_output, .pytest_cache, .ruff_cache, .venv, __pycache__, _build, client/src/ext, coverage, dist, docs/security/crypto-inventory, mochawesome-report, node_modules, test/api/form-data-files, uploads, venv</t>
+          <t>`commit_sha` is HEAD of the checkout at scan time and `source_tree_vs_commit` records whether the scanned source matched it. Because the generated artifacts are committed on top of that source, the SHA recorded inside an artifact is always the parent of the commit that adds the artifact, never that commit itself.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Parsers</t>
+          <t>Excluded</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>cryptography available: True; openssl CLI available: True</t>
+          <t>Directories not scanned: .git, .mypy_cache, .nyc_output, .pytest_cache, .ruff_cache, .venv, __pycache__, _build, client/src/ext, coverage, dist, docs/security/crypto-inventory, mochawesome-report, node_modules, test/api/form-data-files, uploads, venv</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Classes</t>
+          <t>Parsers</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Quantum-vulnerability classes: Quantum-vulnerable (Shor) | Deprecated/weak regardless of PQC | Symmetric — Grover-affected, adequate at ≥256-bit | Protocol/configuration — inherits class of negotiated algorithms | Not applicable (no quantum-relevant primitive)</t>
+          <t>cryptography available: True; openssl CLI available: True</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>Classes</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Quantum-vulnerability classes: Quantum-vulnerable (Shor) | Deprecated/weak regardless of PQC | Symmetric — Grover-affected, adequate at ≥256-bit | Protocol/configuration — inherits class of negotiated algorithms | Not applicable (no quantum-relevant primitive)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>1 = act in Phase 1 (hygiene) or blocks later phases; 2 = Phase 1/2 configuration and TLS work; 3 = track, depends on external party or test-only; 4 = informational, no migration action.</t>
         </is>

</xml_diff>

<commit_message>
crypto-inventory: regenerate artifacts at 4a8aef9
Method text now describes openssl-fallback normalisation and quoted
reference exclusion; counts unchanged (144 rows, 364 files, 64 rules).

Co-Authored-By: Erik Rozi <erik.rozi@cognition.ai>
</commit_message>
<xml_diff>
--- a/docs/security/crypto-inventory/Cryptographic-Inventory.xlsx
+++ b/docs/security/crypto-inventory/Cryptographic-Inventory.xlsx
@@ -18064,7 +18064,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-09-14T22:57:35+00:00</t>
+          <t>2026-09-14T23:09:22+00:00</t>
         </is>
       </c>
     </row>
@@ -18076,7 +18076,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>e426316e995d04bff8ea7cdeb6803e5abce6dec1</t>
+          <t>4a8aef9bcb9200c9255449e08eee0f78a97963d4</t>
         </is>
       </c>
     </row>
@@ -18722,7 +18722,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Secret literals are matched as quoted assignments in any text file and as unquoted scalars only in dotenv, shell, YAML, properties, ini, conf, toml and Dockerfile inputs, where an unquoted value is a literal rather than an identifier; values starting with $, %, {, *, &amp;, &lt; or ( are treated as references or placeholders.</t>
+          <t>Secret literals are matched as quoted assignments in any text file and as unquoted scalars only in dotenv, shell, YAML, properties, ini, conf, toml and Dockerfile inputs, where an unquoted value is a literal rather than an identifier; values starting with $, %, {, *, &amp;, &lt;, ( or [ are treated as references or placeholders whether or not they are quoted (`STIGMAN_DB_PASSWORD="${DB_PASSWORD}"` is a reference, not a literal).</t>
         </is>
       </c>
     </row>
@@ -18758,7 +18758,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Certificate and key files by extension (.cer, .crt, .csr, .der, .jks, .key, .p12, .pem, .pfx) are parsed with `cryptography` or the `openssl` CLI. PEM certificates give subject/issuer attribute types, key algorithm/size, signature algorithm and validity; PEM public keys and unencrypted private keys give key algorithm and size only (public parameters; private components are never read into the output). Files without a PEM block are tried as DER certificate, then DER private key, then DER public key, and get a KEYMAT-DER-* inventory row; keystores and files that parse as none of these get a KEYMAT-FILE-UNPARSED row (priority 2) and are recorded as not parsed. Encrypted keys and unreadable files are recorded as not parsed.</t>
+          <t>Certificate and key files by extension (.cer, .crt, .csr, .der, .jks, .key, .p12, .pem, .pfx) are parsed with `cryptography` or the `openssl` CLI. PEM certificates give subject/issuer attribute types, key algorithm/size, signature algorithm and validity; PEM public keys and unencrypted private keys give key algorithm and size only (public parameters; private components are never read into the output). Files without a PEM block are tried as DER certificate, then DER private key, then DER public key, and get a KEYMAT-DER-* inventory row. The `openssl` fallback normalises its output to the same algorithm labels and sizes as the `cryptography` path (RSA-&lt;bits&gt;, DSA-&lt;bits&gt;, curve name, Ed25519), so RSA/DSA below 2048 bits and SHA-1 signatures are classified weak on either parser; keystores and files that parse as none of these get a KEYMAT-FILE-UNPARSED row (priority 2) and are recorded as not parsed. Encrypted keys and unreadable files are recorded as not parsed.</t>
         </is>
       </c>
     </row>

</xml_diff>